<commit_message>
feat(adtv): backfill ADTV từ vnindex volume — bỏ N/A 24/24 quý (pytest exit=1)
</commit_message>
<xml_diff>
--- a/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
+++ b/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
@@ -17,22 +17,22 @@
     <sheet name="07_Methodology" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Factor_Scores'!$B$5:$G$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Factor_Scores'!$B$5:$G$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="304">
   <si>
     <t>VN-INDEX QUARTERLY QUANT FACTOR WORKBOOK</t>
   </si>
   <si>
-    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-28 10:09:07  |  Source: output/exports/score_*.json</t>
-  </si>
-  <si>
-    <t>49.7</t>
+    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-28 11:09:13  |  Source: output/exports/score_*.json</t>
+  </si>
+  <si>
+    <t>49.4</t>
   </si>
   <si>
     <t>Raw Regime / Label</t>
@@ -44,13 +44,13 @@
     <t>CALIBRATED ACTION</t>
   </si>
   <si>
-    <t>🟠 REDUCE — 35.3</t>
+    <t>🟡 HOLD — 34.5</t>
   </si>
   <si>
     <t>Recommended Equity</t>
   </si>
   <si>
-    <t>20–40% Equities (calibrated)</t>
+    <t>40–60% Equities (calibrated)</t>
   </si>
   <si>
     <t>Percentile Signal</t>
@@ -62,7 +62,7 @@
     <t>Pillar Dispersion</t>
   </si>
   <si>
-    <t>HIGH (σ=14.36)</t>
+    <t>HIGH (σ=13.61)</t>
   </si>
   <si>
     <t>Data As-Of</t>
@@ -185,24 +185,24 @@
     <t>BUY/ACCUMULATE</t>
   </si>
   <si>
+    <t>LOW</t>
+  </si>
+  <si>
     <t>2022-Q2</t>
   </si>
   <si>
     <t>SELL</t>
   </si>
   <si>
+    <t>2022-Q3</t>
+  </si>
+  <si>
+    <t>REDUCE</t>
+  </si>
+  <si>
     <t>HIGH</t>
   </si>
   <si>
-    <t>2022-Q3</t>
-  </si>
-  <si>
-    <t>REDUCE</t>
-  </si>
-  <si>
-    <t>LOW</t>
-  </si>
-  <si>
     <t>2022-Q4</t>
   </si>
   <si>
@@ -713,7 +713,7 @@
     <t>adtv</t>
   </si>
   <si>
-    <t>ADTV data unavailable → neutral score 50</t>
+    <t>ADTV change -11.9% QoQ</t>
   </si>
   <si>
     <t>etf_flow</t>
@@ -728,6 +728,12 @@
     <t>0.00% of Market Cap (YTD in Q)</t>
   </si>
   <si>
+    <t>pillar_components_used</t>
+  </si>
+  <si>
+    <t>3/3 components with data → average over 3</t>
+  </si>
+  <si>
     <t>SIGNAL EFFICACY — DOES THE CALIBRATED ACTION SIGNAL PREDICT NEXT-QUARTER RETURNS?</t>
   </si>
   <si>
@@ -926,7 +932,7 @@
     <t>Data: vnstock (HOSE OHLCV, foreign flows, valuation), yfinance/FRED (DXY, US10Y, USD/JPY), SBV (rates, USD/VND), KBNN (VN yield curve).</t>
   </si>
   <si>
-    <t>Workbook generated at 2026-09-28 10:09:07 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
+    <t>Workbook generated at 2026-09-28 11:09:13 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
   </si>
   <si>
     <t>Disclaimer: for research purposes only. Not financial advice.</t>
@@ -1292,7 +1298,7 @@
                   <c:v>2.59</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6.39</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1467,76 +1473,76 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>61.41</c:v>
+                  <c:v>64.01000000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>52.98</c:v>
+                  <c:v>55.19</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>54.28</c:v>
+                  <c:v>54.94</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>52.83</c:v>
+                  <c:v>52.61</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>63.34</c:v>
+                  <c:v>62.17</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>27.45</c:v>
+                  <c:v>26.12</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>39.08</c:v>
+                  <c:v>35.08</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>17.89</c:v>
+                  <c:v>21.68</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>50.11</c:v>
+                  <c:v>49.98</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>61.36</c:v>
+                  <c:v>55.72</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>66.93000000000001</c:v>
+                  <c:v>66.42</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>43.88</c:v>
+                  <c:v>45.84</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>45.97</c:v>
+                  <c:v>41.76</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>54.51</c:v>
+                  <c:v>54.84</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>50.47</c:v>
+                  <c:v>47.88</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>53</c:v>
+                  <c:v>48.34</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>41.2</c:v>
+                  <c:v>39.85</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>36.51</c:v>
+                  <c:v>39.78</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>49.08</c:v>
+                  <c:v>53.01</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>36.71</c:v>
+                  <c:v>43.29</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>44.52</c:v>
+                  <c:v>38.67</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>14.27</c:v>
+                  <c:v>20.48</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>40.03</c:v>
+                  <c:v>36.76</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>35.27</c:v>
+                  <c:v>34.51</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1646,76 +1652,76 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>61.41</c:v>
+                  <c:v>64.01000000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>52.98</c:v>
+                  <c:v>55.19</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>54.28</c:v>
+                  <c:v>54.94</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>52.83</c:v>
+                  <c:v>52.61</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>59</c:v>
+                  <c:v>60.76</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50.26000000000001</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>52.06</c:v>
+                  <c:v>51.07</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>46.09</c:v>
+                  <c:v>45.8</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>53.65000000000001</c:v>
+                  <c:v>54.29</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>57.02</c:v>
+                  <c:v>56.39</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>58.89</c:v>
+                  <c:v>60.22</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>52.60999999999999</c:v>
+                  <c:v>53.57</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>53.12</c:v>
+                  <c:v>52.15</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>55.39</c:v>
+                  <c:v>56.26</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>54.38000000000001</c:v>
+                  <c:v>54.14</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>55.02</c:v>
+                  <c:v>54.26</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>52.17</c:v>
+                  <c:v>51.77</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>50.97000000000001</c:v>
+                  <c:v>51.63</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>53.79000000000001</c:v>
+                  <c:v>55.24</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>50.94</c:v>
+                  <c:v>52.6</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>52.59</c:v>
+                  <c:v>51.31</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>45.8</c:v>
+                  <c:v>46.38</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>50.96999999999999</c:v>
+                  <c:v>50.12</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>49.73999999999999</c:v>
+                  <c:v>49.35</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1897,7 +1903,7 @@
                   <c:v>1860.01</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1785.11</c:v>
+                  <c:v>1780.68</c:v>
                 </c:pt>
                 <c:pt idx="23">
                   <c:v>0</c:v>
@@ -2766,28 +2772,28 @@
                   <c:v>105.4247172951119</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>104.5586882029319</c:v>
+                  <c:v>104.9050998398039</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>106.2127687154019</c:v>
+                  <c:v>105.9008362111342</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>107.9002453516429</c:v>
+                  <c:v>107.5833569572369</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>114.6192815372562</c:v>
+                  <c:v>114.2826602443579</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>118.8541318652214</c:v>
+                  <c:v>118.5050733909562</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>116.6562006066813</c:v>
+                  <c:v>116.3135971585864</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>120.5335707318928</c:v>
+                  <c:v>120.179579973329</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>120.0481989087403</c:v>
+                  <c:v>119.6670103592256</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2954,7 +2960,7 @@
                   <c:v>156.1144497414892</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>149.8279393003424</c:v>
+                  <c:v>149.4561203249849</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3624,7 +3630,7 @@
         <v>13.58</v>
       </c>
       <c r="F14" s="11">
-        <v>0.2730197024527543</v>
+        <v>0.275177304964539</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>25</v>
@@ -3644,7 +3650,7 @@
         <v>7.44</v>
       </c>
       <c r="F15" s="11">
-        <v>0.149577804583836</v>
+        <v>0.1507598784194529</v>
       </c>
       <c r="G15" s="13" t="s">
         <v>27</v>
@@ -3664,7 +3670,7 @@
         <v>11.5</v>
       </c>
       <c r="F16" s="11">
-        <v>0.2312022517088862</v>
+        <v>0.2330293819655522</v>
       </c>
       <c r="G16" s="12" t="s">
         <v>25</v>
@@ -3684,7 +3690,7 @@
         <v>8.24</v>
       </c>
       <c r="F17" s="11">
-        <v>0.1656614394853237</v>
+        <v>0.1669706180344478</v>
       </c>
       <c r="G17" s="12" t="s">
         <v>25</v>
@@ -3704,7 +3710,7 @@
         <v>2.59</v>
       </c>
       <c r="F18" s="11">
-        <v>0.05207076799356654</v>
+        <v>0.05248226950354609</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>27</v>
@@ -3718,13 +3724,13 @@
         <v>0.1</v>
       </c>
       <c r="D19" s="10">
-        <v>63.94</v>
+        <v>59.97</v>
       </c>
       <c r="E19" s="10">
-        <v>6.39</v>
+        <v>6</v>
       </c>
       <c r="F19" s="11">
-        <v>0.1284680337756333</v>
+        <v>0.121580547112462</v>
       </c>
       <c r="G19" s="12" t="s">
         <v>25</v>
@@ -3739,7 +3745,7 @@
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="10">
-        <v>49.74</v>
+        <v>49.35</v>
       </c>
       <c r="F20" s="11">
         <v>1</v>
@@ -3856,13 +3862,13 @@
         <v>45</v>
       </c>
       <c r="C6" s="10">
-        <v>61.41</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E6" s="10">
-        <v>61.41</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="F6" s="14" t="s">
         <v>33</v>
@@ -3889,7 +3895,7 @@
         <v>8.52</v>
       </c>
       <c r="N6" s="10">
-        <v>5.2</v>
+        <v>7.8</v>
       </c>
       <c r="O6" s="10">
         <v>1191.44</v>
@@ -3906,13 +3912,13 @@
         <v>48</v>
       </c>
       <c r="C7" s="10">
-        <v>52.98</v>
+        <v>55.19</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E7" s="10">
-        <v>52.98</v>
+        <v>55.19</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>33</v>
@@ -3939,7 +3945,7 @@
         <v>3.89</v>
       </c>
       <c r="N7" s="10">
-        <v>5.2</v>
+        <v>7.41</v>
       </c>
       <c r="O7" s="10">
         <v>1408.55</v>
@@ -3956,13 +3962,13 @@
         <v>49</v>
       </c>
       <c r="C8" s="10">
-        <v>54.28</v>
+        <v>54.94</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E8" s="10">
-        <v>54.28</v>
+        <v>54.94</v>
       </c>
       <c r="F8" s="14" t="s">
         <v>33</v>
@@ -3989,7 +3995,7 @@
         <v>3.25</v>
       </c>
       <c r="N8" s="10">
-        <v>5.2</v>
+        <v>5.86</v>
       </c>
       <c r="O8" s="10">
         <v>1342.06</v>
@@ -4006,13 +4012,13 @@
         <v>50</v>
       </c>
       <c r="C9" s="10">
-        <v>52.83</v>
+        <v>52.61</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E9" s="10">
-        <v>52.83</v>
+        <v>52.61</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>33</v>
@@ -4039,7 +4045,7 @@
         <v>3.04</v>
       </c>
       <c r="N9" s="10">
-        <v>5.2</v>
+        <v>4.98</v>
       </c>
       <c r="O9" s="10">
         <v>1498.28</v>
@@ -4056,13 +4062,13 @@
         <v>51</v>
       </c>
       <c r="C10" s="10">
-        <v>59</v>
+        <v>60.76</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E10" s="10">
-        <v>63.34</v>
+        <v>62.17</v>
       </c>
       <c r="F10" s="14" t="s">
         <v>33</v>
@@ -4071,7 +4077,7 @@
         <v>52</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="I10" s="10">
         <v>12.54</v>
@@ -4089,7 +4095,7 @@
         <v>7.91</v>
       </c>
       <c r="N10" s="10">
-        <v>5.2</v>
+        <v>6.96</v>
       </c>
       <c r="O10" s="10">
         <v>1492.15</v>
@@ -4103,25 +4109,25 @@
     </row>
     <row r="11" spans="2:17">
       <c r="B11" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C11" s="10">
-        <v>50.26000000000001</v>
+        <v>50</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E11" s="10">
-        <v>27.45</v>
+        <v>26.12</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="I11" s="10">
         <v>11.73</v>
@@ -4139,7 +4145,7 @@
         <v>2.68</v>
       </c>
       <c r="N11" s="10">
-        <v>4.95</v>
+        <v>4.69</v>
       </c>
       <c r="O11" s="10">
         <v>1197.6</v>
@@ -4156,13 +4162,13 @@
         <v>56</v>
       </c>
       <c r="C12" s="10">
-        <v>52.06</v>
+        <v>51.07</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E12" s="10">
-        <v>39.08</v>
+        <v>35.08</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>57</v>
@@ -4189,7 +4195,7 @@
         <v>7.08</v>
       </c>
       <c r="N12" s="10">
-        <v>4.98</v>
+        <v>3.99</v>
       </c>
       <c r="O12" s="10">
         <v>1132.11</v>
@@ -4206,22 +4212,22 @@
         <v>59</v>
       </c>
       <c r="C13" s="10">
-        <v>46.09</v>
+        <v>45.8</v>
       </c>
       <c r="D13" s="14" t="s">
         <v>57</v>
       </c>
       <c r="E13" s="10">
-        <v>17.89</v>
+        <v>21.68</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I13" s="10">
         <v>9.34</v>
@@ -4239,7 +4245,7 @@
         <v>3.67</v>
       </c>
       <c r="N13" s="10">
-        <v>4.99</v>
+        <v>4.7</v>
       </c>
       <c r="O13" s="10">
         <v>1007.09</v>
@@ -4256,13 +4262,13 @@
         <v>60</v>
       </c>
       <c r="C14" s="10">
-        <v>53.65000000000001</v>
+        <v>54.29</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E14" s="10">
-        <v>50.11</v>
+        <v>49.98</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>33</v>
@@ -4271,7 +4277,7 @@
         <v>33</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I14" s="10">
         <v>12.48</v>
@@ -4289,7 +4295,7 @@
         <v>6.7</v>
       </c>
       <c r="N14" s="10">
-        <v>5.01</v>
+        <v>5.65</v>
       </c>
       <c r="O14" s="10">
         <v>1064.64</v>
@@ -4306,13 +4312,13 @@
         <v>61</v>
       </c>
       <c r="C15" s="10">
-        <v>57.02</v>
+        <v>56.39</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E15" s="10">
-        <v>61.36</v>
+        <v>55.72</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>33</v>
@@ -4321,7 +4327,7 @@
         <v>33</v>
       </c>
       <c r="H15" s="14" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I15" s="10">
         <v>14</v>
@@ -4339,7 +4345,7 @@
         <v>6.86</v>
       </c>
       <c r="N15" s="10">
-        <v>5.02</v>
+        <v>4.39</v>
       </c>
       <c r="O15" s="10">
         <v>1120.18</v>
@@ -4356,13 +4362,13 @@
         <v>62</v>
       </c>
       <c r="C16" s="10">
-        <v>58.89</v>
+        <v>60.22</v>
       </c>
       <c r="D16" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E16" s="10">
-        <v>66.93000000000001</v>
+        <v>66.42</v>
       </c>
       <c r="F16" s="14" t="s">
         <v>63</v>
@@ -4371,7 +4377,7 @@
         <v>52</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="I16" s="10">
         <v>12.77</v>
@@ -4389,7 +4395,7 @@
         <v>6.77</v>
       </c>
       <c r="N16" s="10">
-        <v>5.03</v>
+        <v>6.36</v>
       </c>
       <c r="O16" s="10">
         <v>1154.15</v>
@@ -4406,13 +4412,13 @@
         <v>64</v>
       </c>
       <c r="C17" s="10">
-        <v>52.60999999999999</v>
+        <v>53.57</v>
       </c>
       <c r="D17" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="10">
-        <v>43.88</v>
+        <v>45.84</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>57</v>
@@ -4439,7 +4445,7 @@
         <v>3.36</v>
       </c>
       <c r="N17" s="10">
-        <v>5.04</v>
+        <v>6</v>
       </c>
       <c r="O17" s="10">
         <v>1129.93</v>
@@ -4456,13 +4462,13 @@
         <v>65</v>
       </c>
       <c r="C18" s="10">
-        <v>53.12</v>
+        <v>52.15</v>
       </c>
       <c r="D18" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E18" s="10">
-        <v>45.97</v>
+        <v>41.76</v>
       </c>
       <c r="F18" s="14" t="s">
         <v>57</v>
@@ -4471,7 +4477,7 @@
         <v>33</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I18" s="10">
         <v>16.31</v>
@@ -4489,7 +4495,7 @@
         <v>6.76</v>
       </c>
       <c r="N18" s="10">
-        <v>5.05</v>
+        <v>4.08</v>
       </c>
       <c r="O18" s="10">
         <v>1284.09</v>
@@ -4506,13 +4512,13 @@
         <v>66</v>
       </c>
       <c r="C19" s="10">
-        <v>55.39</v>
+        <v>56.26</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E19" s="10">
-        <v>54.51</v>
+        <v>54.84</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>33</v>
@@ -4521,7 +4527,7 @@
         <v>33</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I19" s="10">
         <v>14.83</v>
@@ -4539,7 +4545,7 @@
         <v>6.96</v>
       </c>
       <c r="N19" s="10">
-        <v>5.05</v>
+        <v>5.92</v>
       </c>
       <c r="O19" s="10">
         <v>1245.32</v>
@@ -4556,22 +4562,22 @@
         <v>67</v>
       </c>
       <c r="C20" s="10">
-        <v>54.38000000000001</v>
+        <v>54.14</v>
       </c>
       <c r="D20" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E20" s="10">
-        <v>50.47</v>
+        <v>47.88</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="G20" s="14" t="s">
         <v>33</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="I20" s="10">
         <v>14.55</v>
@@ -4589,7 +4595,7 @@
         <v>7.53</v>
       </c>
       <c r="N20" s="10">
-        <v>5.06</v>
+        <v>4.82</v>
       </c>
       <c r="O20" s="10">
         <v>1287.94</v>
@@ -4606,22 +4612,22 @@
         <v>68</v>
       </c>
       <c r="C21" s="10">
-        <v>55.02</v>
+        <v>54.26</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E21" s="10">
-        <v>53</v>
+        <v>48.34</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="G21" s="14" t="s">
         <v>33</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I21" s="10">
         <v>16.84</v>
@@ -4639,7 +4645,7 @@
         <v>4.73</v>
       </c>
       <c r="N21" s="10">
-        <v>5.07</v>
+        <v>4.31</v>
       </c>
       <c r="O21" s="10">
         <v>1266.78</v>
@@ -4656,19 +4662,19 @@
         <v>69</v>
       </c>
       <c r="C22" s="10">
-        <v>52.17</v>
+        <v>51.77</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E22" s="10">
-        <v>41.2</v>
+        <v>39.85</v>
       </c>
       <c r="F22" s="14" t="s">
         <v>57</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="H22" s="14" t="s">
         <v>46</v>
@@ -4689,7 +4695,7 @@
         <v>7.01</v>
       </c>
       <c r="N22" s="10">
-        <v>5.07</v>
+        <v>4.67</v>
       </c>
       <c r="O22" s="10">
         <v>1306.86</v>
@@ -4706,22 +4712,22 @@
         <v>70</v>
       </c>
       <c r="C23" s="10">
-        <v>50.97000000000001</v>
+        <v>51.63</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E23" s="10">
-        <v>36.51</v>
+        <v>39.78</v>
       </c>
       <c r="F23" s="14" t="s">
         <v>57</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="H23" s="14" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I23" s="10">
         <v>14.58</v>
@@ -4739,7 +4745,7 @@
         <v>4.67</v>
       </c>
       <c r="N23" s="10">
-        <v>5.07</v>
+        <v>5.73</v>
       </c>
       <c r="O23" s="10">
         <v>1376.07</v>
@@ -4756,13 +4762,13 @@
         <v>71</v>
       </c>
       <c r="C24" s="10">
-        <v>53.79000000000001</v>
+        <v>55.24</v>
       </c>
       <c r="D24" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E24" s="10">
-        <v>49.08</v>
+        <v>53.01</v>
       </c>
       <c r="F24" s="14" t="s">
         <v>33</v>
@@ -4789,7 +4795,7 @@
         <v>6.97</v>
       </c>
       <c r="N24" s="10">
-        <v>5.25</v>
+        <v>6.7</v>
       </c>
       <c r="O24" s="10">
         <v>1661.7</v>
@@ -4806,22 +4812,22 @@
         <v>72</v>
       </c>
       <c r="C25" s="10">
-        <v>50.94</v>
+        <v>52.6</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E25" s="10">
-        <v>36.71</v>
+        <v>43.29</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>57</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I25" s="10">
         <v>13.06</v>
@@ -4839,7 +4845,7 @@
         <v>6.92</v>
       </c>
       <c r="N25" s="10">
-        <v>5.25</v>
+        <v>6.91</v>
       </c>
       <c r="O25" s="10">
         <v>1784.49</v>
@@ -4856,22 +4862,22 @@
         <v>73</v>
       </c>
       <c r="C26" s="10">
-        <v>52.59</v>
+        <v>51.31</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E26" s="10">
-        <v>44.52</v>
+        <v>38.67</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>57</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I26" s="10">
         <v>16.02</v>
@@ -4889,7 +4895,7 @@
         <v>4.89</v>
       </c>
       <c r="N26" s="10">
-        <v>5.25</v>
+        <v>3.97</v>
       </c>
       <c r="O26" s="10">
         <v>1674.49</v>
@@ -4906,22 +4912,22 @@
         <v>74</v>
       </c>
       <c r="C27" s="10">
-        <v>45.8</v>
+        <v>46.38</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="10">
-        <v>14.27</v>
+        <v>20.48</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G27" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I27" s="10">
         <v>11.71</v>
@@ -4939,7 +4945,7 @@
         <v>7</v>
       </c>
       <c r="N27" s="10">
-        <v>5.25</v>
+        <v>5.83</v>
       </c>
       <c r="O27" s="10">
         <v>1860.01</v>
@@ -4948,7 +4954,7 @@
         <v>0.1107919426213355</v>
       </c>
       <c r="Q27" s="11">
-        <v>-0.04026860070644789</v>
+        <v>-0.0426503083316756</v>
       </c>
     </row>
     <row r="28" spans="2:17">
@@ -4956,22 +4962,22 @@
         <v>75</v>
       </c>
       <c r="C28" s="10">
-        <v>50.96999999999999</v>
+        <v>50.12</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E28" s="10">
-        <v>40.03</v>
+        <v>36.76</v>
       </c>
       <c r="F28" s="14" t="s">
         <v>57</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I28" s="10">
         <v>14.41</v>
@@ -4989,13 +4995,13 @@
         <v>6.86</v>
       </c>
       <c r="N28" s="10">
-        <v>5.26</v>
+        <v>4.41</v>
       </c>
       <c r="O28" s="10">
-        <v>1785.11</v>
+        <v>1780.68</v>
       </c>
       <c r="P28" s="11">
-        <v>-0.04026860070644789</v>
+        <v>-0.0426503083316756</v>
       </c>
       <c r="Q28" s="14" t="s">
         <v>47</v>
@@ -5006,22 +5012,22 @@
         <v>76</v>
       </c>
       <c r="C29" s="10">
-        <v>49.73999999999999</v>
+        <v>49.35</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E29" s="10">
-        <v>35.27</v>
+        <v>34.51</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I29" s="10">
         <v>13.58</v>
@@ -5039,7 +5045,7 @@
         <v>2.59</v>
       </c>
       <c r="N29" s="10">
-        <v>6.39</v>
+        <v>6</v>
       </c>
       <c r="O29" s="14" t="s">
         <v>47</v>
@@ -5527,7 +5533,7 @@
         <v>51</v>
       </c>
       <c r="H40" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I40" s="7" t="s">
         <v>56</v>
@@ -7220,7 +7226,7 @@
   <sheetPr>
     <tabColor rgb="FFF97316"/>
   </sheetPr>
-  <dimension ref="B2:G30"/>
+  <dimension ref="B2:G31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.7109375" customWidth="1"/>
@@ -7715,11 +7721,11 @@
       <c r="E28" s="18" t="s">
         <v>229</v>
       </c>
-      <c r="F28" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="G28" s="13" t="s">
-        <v>193</v>
+      <c r="F28" s="10">
+        <v>38</v>
+      </c>
+      <c r="G28" s="17" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="2:7">
@@ -7762,9 +7768,29 @@
         <v>187</v>
       </c>
     </row>
+    <row r="31" spans="2:7">
+      <c r="B31" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C31" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="G31" s="17" t="s">
+        <v>187</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B5:G30"/>
-  <conditionalFormatting sqref="F6:F30">
+  <autoFilter ref="B5:G31"/>
+  <conditionalFormatting sqref="F6:F31">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -7801,17 +7827,17 @@
   <sheetData>
     <row r="2" spans="2:3">
       <c r="B2" s="1" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="2:3">
       <c r="B3" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C5" s="14">
         <v>22</v>
@@ -7819,39 +7845,39 @@
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="4" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C6" s="16">
-        <v>0.004156386627439163</v>
+        <v>0.05191697881001582</v>
       </c>
     </row>
     <row r="7" spans="2:3">
       <c r="B7" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C7" s="16">
-        <v>0.01637492941840768</v>
+        <v>0.05138339920948617</v>
       </c>
     </row>
     <row r="8" spans="2:3">
       <c r="B8" s="4" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C8" s="16">
-        <v>0.02840623638565849</v>
+        <v>0.03936735417591136</v>
       </c>
     </row>
     <row r="9" spans="2:3">
       <c r="B9" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C9" s="16">
-        <v>0.09203839638622249</v>
+        <v>0.07735742518351214</v>
       </c>
     </row>
     <row r="10" spans="2:3">
       <c r="B10" s="4" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C10" s="11">
         <v>0.5</v>
@@ -7859,7 +7885,7 @@
     </row>
     <row r="11" spans="2:3">
       <c r="B11" s="4" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C11" s="11">
         <v>0.5454545454545454</v>
@@ -7867,64 +7893,64 @@
     </row>
     <row r="12" spans="2:3">
       <c r="B12" s="4" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C12" s="11">
-        <v>0.2004819890874032</v>
+        <v>0.1966701035922562</v>
       </c>
     </row>
     <row r="13" spans="2:3">
       <c r="B13" s="4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C13" s="11">
-        <v>0.2503907960980185</v>
+        <v>0.249486451502519</v>
       </c>
     </row>
     <row r="14" spans="2:3">
       <c r="B14" s="4" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C14" s="11">
-        <v>0.4982793930034239</v>
+        <v>0.4945612032498485</v>
       </c>
     </row>
     <row r="15" spans="2:3">
       <c r="B15" s="4" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C15" s="10">
-        <v>0.4656941087978428</v>
+        <v>0.4590638734741476</v>
       </c>
     </row>
     <row r="16" spans="2:3">
       <c r="B16" s="4" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C16" s="10">
-        <v>0.4801617850137476</v>
+        <v>0.4775014136300051</v>
       </c>
     </row>
     <row r="18" spans="2:12">
       <c r="B18" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="19" spans="2:12">
       <c r="B19" s="7" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="20" spans="2:12">
@@ -7949,16 +7975,16 @@
         <v>33</v>
       </c>
       <c r="C21" s="14">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D21" s="11">
-        <v>0.02325036242226524</v>
+        <v>0.02672711655939455</v>
       </c>
       <c r="E21" s="11">
-        <v>0.03163927438071323</v>
+        <v>0.0342241351620467</v>
       </c>
       <c r="F21" s="11">
-        <v>0.6363636363636364</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="22" spans="2:12">
@@ -7966,30 +7992,30 @@
         <v>57</v>
       </c>
       <c r="C22" s="14">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D22" s="11">
-        <v>0.04364110592335368</v>
+        <v>0.03563307545264917</v>
       </c>
       <c r="E22" s="11">
-        <v>0.05295900096414319</v>
+        <v>0.03163927438071323</v>
       </c>
       <c r="F22" s="11">
-        <v>0.5714285714285714</v>
+        <v>0.5555555555555556</v>
       </c>
     </row>
     <row r="23" spans="2:12">
       <c r="B23" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C23" s="14">
         <v>3</v>
       </c>
       <c r="D23" s="11">
-        <v>-0.01260270879374577</v>
+        <v>-0.01339661133548834</v>
       </c>
       <c r="E23" s="11">
-        <v>-0.04026860070644789</v>
+        <v>-0.0426503083316756</v>
       </c>
       <c r="F23" s="11">
         <v>0.3333333333333333</v>
@@ -7997,7 +8023,7 @@
     </row>
     <row r="25" spans="2:12">
       <c r="B25" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="26" spans="2:12">
@@ -8005,34 +8031,34 @@
         <v>36</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>40</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="H26" s="7" t="s">
         <v>44</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="27" spans="2:12">
@@ -8040,7 +8066,7 @@
         <v>45</v>
       </c>
       <c r="C27" s="10">
-        <v>61.41</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>33</v>
@@ -8049,7 +8075,7 @@
         <v>0.5</v>
       </c>
       <c r="F27" s="10">
-        <v>61.41</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="G27" s="14" t="s">
         <v>33</v>
@@ -8061,7 +8087,7 @@
         <v>0.0911124353723225</v>
       </c>
       <c r="J27" s="17" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K27" s="10">
         <v>109.1112435372323</v>
@@ -8075,7 +8101,7 @@
         <v>48</v>
       </c>
       <c r="C28" s="10">
-        <v>52.98</v>
+        <v>55.19</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>33</v>
@@ -8084,7 +8110,7 @@
         <v>0.5</v>
       </c>
       <c r="F28" s="10">
-        <v>52.98</v>
+        <v>55.19</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>33</v>
@@ -8096,7 +8122,7 @@
         <v>-0.02360228603883424</v>
       </c>
       <c r="J28" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K28" s="10">
         <v>106.5359687572136</v>
@@ -8110,7 +8136,7 @@
         <v>49</v>
       </c>
       <c r="C29" s="10">
-        <v>54.28</v>
+        <v>54.94</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>33</v>
@@ -8119,7 +8145,7 @@
         <v>0.5</v>
       </c>
       <c r="F29" s="10">
-        <v>54.28</v>
+        <v>54.94</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>33</v>
@@ -8131,7 +8157,7 @@
         <v>0.05820157071963994</v>
       </c>
       <c r="J29" s="17" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K29" s="10">
         <v>112.7365294770219</v>
@@ -8145,7 +8171,7 @@
         <v>50</v>
       </c>
       <c r="C30" s="10">
-        <v>52.83</v>
+        <v>52.61</v>
       </c>
       <c r="D30" s="14" t="s">
         <v>33</v>
@@ -8154,7 +8180,7 @@
         <v>0.5</v>
       </c>
       <c r="F30" s="10">
-        <v>52.83</v>
+        <v>52.61</v>
       </c>
       <c r="G30" s="14" t="s">
         <v>33</v>
@@ -8166,7 +8192,7 @@
         <v>-0.002045679045305226</v>
       </c>
       <c r="J30" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K30" s="10">
         <v>112.5059067210303</v>
@@ -8180,7 +8206,7 @@
         <v>51</v>
       </c>
       <c r="C31" s="10">
-        <v>63.34</v>
+        <v>62.17</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>33</v>
@@ -8189,7 +8215,7 @@
         <v>0.5</v>
       </c>
       <c r="F31" s="10">
-        <v>59</v>
+        <v>60.76</v>
       </c>
       <c r="G31" s="14" t="s">
         <v>33</v>
@@ -8201,7 +8227,7 @@
         <v>-0.09869986261434849</v>
       </c>
       <c r="J31" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K31" s="10">
         <v>101.4015891843619</v>
@@ -8212,19 +8238,19 @@
     </row>
     <row r="32" spans="2:12">
       <c r="B32" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C32" s="10">
-        <v>27.45</v>
+        <v>26.12</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E32" s="9">
         <v>0.1</v>
       </c>
       <c r="F32" s="10">
-        <v>50.26000000000001</v>
+        <v>50</v>
       </c>
       <c r="G32" s="14" t="s">
         <v>33</v>
@@ -8236,7 +8262,7 @@
         <v>-0.005468436873747495</v>
       </c>
       <c r="J32" s="17" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K32" s="10">
         <v>100.8470809950096</v>
@@ -8250,7 +8276,7 @@
         <v>56</v>
       </c>
       <c r="C33" s="10">
-        <v>39.08</v>
+        <v>35.08</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>57</v>
@@ -8259,7 +8285,7 @@
         <v>0.3</v>
       </c>
       <c r="F33" s="10">
-        <v>52.06</v>
+        <v>51.07</v>
       </c>
       <c r="G33" s="14" t="s">
         <v>33</v>
@@ -8271,7 +8297,7 @@
         <v>-0.03312928955666848</v>
       </c>
       <c r="J33" s="17" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K33" s="10">
         <v>97.50608884778109</v>
@@ -8285,16 +8311,16 @@
         <v>59</v>
       </c>
       <c r="C34" s="10">
-        <v>17.89</v>
+        <v>21.68</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E34" s="9">
         <v>0.1</v>
       </c>
       <c r="F34" s="10">
-        <v>46.09</v>
+        <v>45.8</v>
       </c>
       <c r="G34" s="14" t="s">
         <v>57</v>
@@ -8306,7 +8332,7 @@
         <v>0.005714484306268553</v>
       </c>
       <c r="J34" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K34" s="10">
         <v>98.06328586226736</v>
@@ -8320,7 +8346,7 @@
         <v>60</v>
       </c>
       <c r="C35" s="10">
-        <v>50.11</v>
+        <v>49.98</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>33</v>
@@ -8329,7 +8355,7 @@
         <v>0.5</v>
       </c>
       <c r="F35" s="10">
-        <v>53.65000000000001</v>
+        <v>54.29</v>
       </c>
       <c r="G35" s="14" t="s">
         <v>33</v>
@@ -8340,8 +8366,8 @@
       <c r="I35" s="11">
         <v>0.02608393447550339</v>
       </c>
-      <c r="J35" s="17" t="s">
-        <v>263</v>
+      <c r="J35" s="13" t="s">
+        <v>266</v>
       </c>
       <c r="K35" s="10">
         <v>100.6211621851513</v>
@@ -8355,7 +8381,7 @@
         <v>61</v>
       </c>
       <c r="C36" s="10">
-        <v>61.36</v>
+        <v>55.72</v>
       </c>
       <c r="D36" s="14" t="s">
         <v>33</v>
@@ -8364,7 +8390,7 @@
         <v>0.5</v>
       </c>
       <c r="F36" s="10">
-        <v>57.02</v>
+        <v>56.39</v>
       </c>
       <c r="G36" s="14" t="s">
         <v>33</v>
@@ -8376,7 +8402,7 @@
         <v>0.01516274170222642</v>
       </c>
       <c r="J36" s="17" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K36" s="10">
         <v>102.1468548771426</v>
@@ -8390,7 +8416,7 @@
         <v>62</v>
       </c>
       <c r="C37" s="10">
-        <v>66.93000000000001</v>
+        <v>66.42</v>
       </c>
       <c r="D37" s="14" t="s">
         <v>63</v>
@@ -8399,7 +8425,7 @@
         <v>0.775</v>
       </c>
       <c r="F37" s="10">
-        <v>58.89</v>
+        <v>60.22</v>
       </c>
       <c r="G37" s="14" t="s">
         <v>33</v>
@@ -8411,7 +8437,7 @@
         <v>-0.01626348394922673</v>
       </c>
       <c r="J37" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K37" s="10">
         <v>100.4855911423842</v>
@@ -8425,7 +8451,7 @@
         <v>64</v>
       </c>
       <c r="C38" s="10">
-        <v>43.88</v>
+        <v>45.84</v>
       </c>
       <c r="D38" s="14" t="s">
         <v>57</v>
@@ -8434,7 +8460,7 @@
         <v>0.3</v>
       </c>
       <c r="F38" s="10">
-        <v>52.60999999999999</v>
+        <v>53.57</v>
       </c>
       <c r="G38" s="14" t="s">
         <v>33</v>
@@ -8446,7 +8472,7 @@
         <v>0.04092996911313089</v>
       </c>
       <c r="J38" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K38" s="10">
         <v>104.5984632841567</v>
@@ -8460,7 +8486,7 @@
         <v>65</v>
       </c>
       <c r="C39" s="10">
-        <v>45.97</v>
+        <v>41.76</v>
       </c>
       <c r="D39" s="14" t="s">
         <v>57</v>
@@ -8469,7 +8495,7 @@
         <v>0.3</v>
       </c>
       <c r="F39" s="10">
-        <v>53.12</v>
+        <v>52.15</v>
       </c>
       <c r="G39" s="14" t="s">
         <v>33</v>
@@ -8481,7 +8507,7 @@
         <v>-0.009057776324089427</v>
       </c>
       <c r="J39" s="17" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K39" s="10">
         <v>103.6510337998853</v>
@@ -8495,7 +8521,7 @@
         <v>66</v>
       </c>
       <c r="C40" s="10">
-        <v>54.51</v>
+        <v>54.84</v>
       </c>
       <c r="D40" s="14" t="s">
         <v>33</v>
@@ -8504,7 +8530,7 @@
         <v>0.5</v>
       </c>
       <c r="F40" s="10">
-        <v>55.39</v>
+        <v>56.26</v>
       </c>
       <c r="G40" s="14" t="s">
         <v>33</v>
@@ -8516,7 +8542,7 @@
         <v>0.01711206758102335</v>
       </c>
       <c r="J40" s="17" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K40" s="10">
         <v>105.4247172951119</v>
@@ -8530,16 +8556,16 @@
         <v>67</v>
       </c>
       <c r="C41" s="10">
-        <v>50.47</v>
+        <v>47.88</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="E41" s="9">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="F41" s="10">
-        <v>54.38000000000001</v>
+        <v>54.14</v>
       </c>
       <c r="G41" s="14" t="s">
         <v>33</v>
@@ -8548,13 +8574,13 @@
         <v>-0.01642933677034653</v>
       </c>
       <c r="I41" s="11">
-        <v>-0.008214668385173263</v>
-      </c>
-      <c r="J41" s="13" t="s">
-        <v>264</v>
+        <v>-0.004928801031103957</v>
+      </c>
+      <c r="J41" s="17" t="s">
+        <v>265</v>
       </c>
       <c r="K41" s="10">
-        <v>104.5586882029319</v>
+        <v>104.9050998398039</v>
       </c>
       <c r="L41" s="10">
         <v>106.3234405425367</v>
@@ -8565,16 +8591,16 @@
         <v>68</v>
       </c>
       <c r="C42" s="10">
-        <v>53</v>
+        <v>48.34</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="E42" s="9">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="F42" s="10">
-        <v>55.02</v>
+        <v>54.26</v>
       </c>
       <c r="G42" s="14" t="s">
         <v>33</v>
@@ -8583,13 +8609,13 @@
         <v>0.03163927438071323</v>
       </c>
       <c r="I42" s="11">
-        <v>0.01581963719035662</v>
-      </c>
-      <c r="J42" s="17" t="s">
-        <v>263</v>
+        <v>0.00949178231421397</v>
+      </c>
+      <c r="J42" s="13" t="s">
+        <v>266</v>
       </c>
       <c r="K42" s="10">
-        <v>106.2127687154019</v>
+        <v>105.9008362111342</v>
       </c>
       <c r="L42" s="10">
         <v>109.6874370509635</v>
@@ -8600,7 +8626,7 @@
         <v>69</v>
       </c>
       <c r="C43" s="10">
-        <v>41.2</v>
+        <v>39.85</v>
       </c>
       <c r="D43" s="14" t="s">
         <v>57</v>
@@ -8609,7 +8635,7 @@
         <v>0.3</v>
       </c>
       <c r="F43" s="10">
-        <v>52.17</v>
+        <v>51.77</v>
       </c>
       <c r="G43" s="14" t="s">
         <v>33</v>
@@ -8621,10 +8647,10 @@
         <v>0.01588770028924296</v>
       </c>
       <c r="J43" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K43" s="10">
-        <v>107.9002453516429</v>
+        <v>107.5833569572369</v>
       </c>
       <c r="L43" s="10">
         <v>115.4963741354999</v>
@@ -8635,7 +8661,7 @@
         <v>70</v>
       </c>
       <c r="C44" s="10">
-        <v>36.51</v>
+        <v>39.78</v>
       </c>
       <c r="D44" s="14" t="s">
         <v>57</v>
@@ -8644,7 +8670,7 @@
         <v>0.3</v>
       </c>
       <c r="F44" s="10">
-        <v>50.97000000000001</v>
+        <v>51.63</v>
       </c>
       <c r="G44" s="14" t="s">
         <v>33</v>
@@ -8656,10 +8682,10 @@
         <v>0.0622708147114609</v>
       </c>
       <c r="J44" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K44" s="10">
-        <v>114.6192815372562</v>
+        <v>114.2826602443579</v>
       </c>
       <c r="L44" s="10">
         <v>139.4698851809575</v>
@@ -8670,7 +8696,7 @@
         <v>71</v>
       </c>
       <c r="C45" s="10">
-        <v>49.08</v>
+        <v>53.01</v>
       </c>
       <c r="D45" s="14" t="s">
         <v>33</v>
@@ -8679,7 +8705,7 @@
         <v>0.5</v>
       </c>
       <c r="F45" s="10">
-        <v>53.79000000000001</v>
+        <v>55.24</v>
       </c>
       <c r="G45" s="14" t="s">
         <v>33</v>
@@ -8690,11 +8716,11 @@
       <c r="I45" s="11">
         <v>0.03694710236504783</v>
       </c>
-      <c r="J45" s="13" t="s">
-        <v>264</v>
+      <c r="J45" s="17" t="s">
+        <v>265</v>
       </c>
       <c r="K45" s="10">
-        <v>118.8541318652214</v>
+        <v>118.5050733909562</v>
       </c>
       <c r="L45" s="10">
         <v>149.7759014302021</v>
@@ -8705,7 +8731,7 @@
         <v>72</v>
       </c>
       <c r="C46" s="10">
-        <v>36.71</v>
+        <v>43.29</v>
       </c>
       <c r="D46" s="14" t="s">
         <v>57</v>
@@ -8714,7 +8740,7 @@
         <v>0.3</v>
       </c>
       <c r="F46" s="10">
-        <v>50.94</v>
+        <v>52.6</v>
       </c>
       <c r="G46" s="14" t="s">
         <v>33</v>
@@ -8726,10 +8752,10 @@
         <v>-0.01849267858043475</v>
       </c>
       <c r="J46" s="17" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K46" s="10">
-        <v>116.6562006066813</v>
+        <v>116.3135971585864</v>
       </c>
       <c r="L46" s="10">
         <v>140.5433760827234</v>
@@ -8740,7 +8766,7 @@
         <v>73</v>
       </c>
       <c r="C47" s="10">
-        <v>44.52</v>
+        <v>38.67</v>
       </c>
       <c r="D47" s="14" t="s">
         <v>57</v>
@@ -8749,7 +8775,7 @@
         <v>0.3</v>
       </c>
       <c r="F47" s="10">
-        <v>52.59</v>
+        <v>51.31</v>
       </c>
       <c r="G47" s="14" t="s">
         <v>33</v>
@@ -8761,10 +8787,10 @@
         <v>0.03323758278640065</v>
       </c>
       <c r="J47" s="13" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K47" s="10">
-        <v>120.5335707318928</v>
+        <v>120.179579973329</v>
       </c>
       <c r="L47" s="10">
         <v>156.1144497414892</v>
@@ -8775,39 +8801,39 @@
         <v>74</v>
       </c>
       <c r="C48" s="10">
-        <v>14.27</v>
+        <v>20.48</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E48" s="9">
         <v>0.1</v>
       </c>
       <c r="F48" s="10">
-        <v>45.8</v>
+        <v>46.38</v>
       </c>
       <c r="G48" s="14" t="s">
         <v>57</v>
       </c>
       <c r="H48" s="11">
-        <v>-0.04026860070644789</v>
+        <v>-0.0426503083316756</v>
       </c>
       <c r="I48" s="11">
-        <v>-0.004026860070644789</v>
+        <v>-0.004265030833167561</v>
       </c>
       <c r="J48" s="17" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="K48" s="10">
-        <v>120.0481989087403</v>
+        <v>119.6670103592256</v>
       </c>
       <c r="L48" s="10">
-        <v>149.8279393003424</v>
+        <v>149.4561203249849</v>
       </c>
     </row>
     <row r="69" spans="2:2">
       <c r="B69" s="19" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -8833,7 +8859,7 @@
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="2:5">
@@ -8894,104 +8920,104 @@
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="2:5">
       <c r="B14" s="7" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="14" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="14" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17" spans="2:9">
       <c r="B17" s="14" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="18" spans="2:9">
       <c r="B18" s="14" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="19" spans="2:9">
       <c r="B19" s="14" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="21" spans="2:9">
       <c r="B21" s="6" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="22" spans="2:9">
       <c r="B22" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D22" s="19"/>
       <c r="E22" s="19"/>
@@ -9002,10 +9028,10 @@
     </row>
     <row r="23" spans="2:9">
       <c r="B23" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D23" s="19"/>
       <c r="E23" s="19"/>
@@ -9016,10 +9042,10 @@
     </row>
     <row r="24" spans="2:9">
       <c r="B24" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D24" s="19"/>
       <c r="E24" s="19"/>
@@ -9030,10 +9056,10 @@
     </row>
     <row r="25" spans="2:9">
       <c r="B25" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D25" s="19"/>
       <c r="E25" s="19"/>
@@ -9044,10 +9070,10 @@
     </row>
     <row r="26" spans="2:9">
       <c r="B26" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D26" s="19"/>
       <c r="E26" s="19"/>
@@ -9058,10 +9084,10 @@
     </row>
     <row r="27" spans="2:9">
       <c r="B27" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D27" s="19"/>
       <c r="E27" s="19"/>
@@ -9072,10 +9098,10 @@
     </row>
     <row r="28" spans="2:9">
       <c r="B28" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D28" s="19"/>
       <c r="E28" s="19"/>
@@ -9086,10 +9112,10 @@
     </row>
     <row r="29" spans="2:9">
       <c r="B29" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D29" s="19"/>
       <c r="E29" s="19"/>
@@ -9100,10 +9126,10 @@
     </row>
     <row r="30" spans="2:9">
       <c r="B30" s="14" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="D30" s="19"/>
       <c r="E30" s="19"/>

</xml_diff>

<commit_message>
feat(adtv): backfill ADTV từ vnindex volume — bỏ N/A 24/24 quý (market_structure)
</commit_message>
<xml_diff>
--- a/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
+++ b/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
@@ -29,7 +29,7 @@
     <t>VN-INDEX QUARTERLY QUANT FACTOR WORKBOOK</t>
   </si>
   <si>
-    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-28 11:15:45  |  Source: output/exports/score_*.json</t>
+    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-28 11:17:50  |  Source: output/exports/score_*.json</t>
   </si>
   <si>
     <t>49.4</t>
@@ -932,7 +932,7 @@
     <t>Data: vnstock (HOSE OHLCV, foreign flows, valuation), yfinance/FRED (DXY, US10Y, USD/JPY), SBV (rates, USD/VND), KBNN (VN yield curve).</t>
   </si>
   <si>
-    <t>Workbook generated at 2026-09-28 11:15:45 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
+    <t>Workbook generated at 2026-09-28 11:17:50 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
   </si>
   <si>
     <t>Disclaimer: for research purposes only. Not financial advice.</t>

</xml_diff>

<commit_message>
feat(market-data): backfill bonds full-history + M2 ADB/GSO + PE/PB/EYG Z-score — bỏ N/A
</commit_message>
<xml_diff>
--- a/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
+++ b/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
@@ -29,7 +29,7 @@
     <t>VN-INDEX QUARTERLY QUANT FACTOR WORKBOOK</t>
   </si>
   <si>
-    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-28 12:05:04  |  Source: output/exports/score_*.json</t>
+    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-28 12:11:45  |  Source: output/exports/score_*.json</t>
   </si>
   <si>
     <t>47.3</t>
@@ -935,7 +935,7 @@
     <t>Data: vnstock (HOSE OHLCV, foreign flows, valuation), yfinance/FRED (DXY, US10Y, USD/JPY), SBV (rates, USD/VND), KBNN (VN yield curve).</t>
   </si>
   <si>
-    <t>Workbook generated at 2026-09-28 12:05:04 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
+    <t>Workbook generated at 2026-09-28 12:11:45 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
   </si>
   <si>
     <t>Disclaimer: for research purposes only. Not financial advice.</t>

</xml_diff>

<commit_message>
feat(flows): backfill foreign flows 2018→nay — bỏ N/A 5 quý + sửa expanding stats nhiễm MC rác
</commit_message>
<xml_diff>
--- a/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
+++ b/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
@@ -24,15 +24,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="306">
   <si>
     <t>VN-INDEX QUARTERLY QUANT FACTOR WORKBOOK</t>
   </si>
   <si>
-    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-28 12:11:45  |  Source: output/exports/score_*.json</t>
-  </si>
-  <si>
-    <t>47.3</t>
+    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-28 15:48:37  |  Source: output/exports/score_*.json</t>
+  </si>
+  <si>
+    <t>47.2</t>
   </si>
   <si>
     <t>Raw Regime / Label</t>
@@ -44,7 +44,7 @@
     <t>CALIBRATED ACTION</t>
   </si>
   <si>
-    <t>🔴 SELL — 28.2</t>
+    <t>🔴 SELL — 29.4</t>
   </si>
   <si>
     <t>Recommended Equity</t>
@@ -62,7 +62,7 @@
     <t>Pillar Dispersion</t>
   </si>
   <si>
-    <t>MEDIUM (σ=13.47)</t>
+    <t>MEDIUM (σ=13.67)</t>
   </si>
   <si>
     <t>Data As-Of</t>
@@ -209,6 +209,9 @@
     <t>2023-Q1</t>
   </si>
   <si>
+    <t>BUY/ACCUMULATE</t>
+  </si>
+  <si>
     <t>2023-Q2</t>
   </si>
   <si>
@@ -626,7 +629,7 @@
     <t>nff_ex_etf</t>
   </si>
   <si>
-    <t>Z = 0.21 (Neutral)</t>
+    <t>Z = -0.05 (Neutral)</t>
   </si>
   <si>
     <t>-0.16% of Market Cap (YTD in Q)</t>
@@ -722,7 +725,7 @@
     <t>etf_flow</t>
   </si>
   <si>
-    <t>Z = -0.21 (Neutral)</t>
+    <t>Z = -0.12 (Neutral)</t>
   </si>
   <si>
     <t>etf_flow_q_ytd</t>
@@ -935,7 +938,7 @@
     <t>Data: vnstock (HOSE OHLCV, foreign flows, valuation), yfinance/FRED (DXY, US10Y, USD/JPY), SBV (rates, USD/VND), KBNN (VN yield curve).</t>
   </si>
   <si>
-    <t>Workbook generated at 2026-09-28 12:11:45 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
+    <t>Workbook generated at 2026-09-28 15:48:37 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
   </si>
   <si>
     <t>Disclaimer: for research purposes only. Not financial advice.</t>
@@ -1289,7 +1292,7 @@
                   <c:v>14.48</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.44</c:v>
+                  <c:v>7.28</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>8.57</c:v>
@@ -1301,7 +1304,7 @@
                   <c:v>2.59</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6</c:v>
+                  <c:v>6.04</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1476,76 +1479,76 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>70.13</c:v>
+                  <c:v>68.64</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>61.25</c:v>
+                  <c:v>60.11</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>60.67</c:v>
+                  <c:v>60.26</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>58.17</c:v>
+                  <c:v>57.42</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>46.08</c:v>
+                  <c:v>45.35</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>11.75</c:v>
+                  <c:v>11.29</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>43.58</c:v>
+                  <c:v>46.77</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>22.14</c:v>
+                  <c:v>20.65</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>52.25</c:v>
+                  <c:v>57.76</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>52.96</c:v>
+                  <c:v>54.48</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>51.43</c:v>
+                  <c:v>51.08</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>32.74</c:v>
+                  <c:v>31.03</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>30.74</c:v>
+                  <c:v>29.31</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>46.17</c:v>
+                  <c:v>44.81</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>40.55</c:v>
+                  <c:v>37.27</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>41.03</c:v>
+                  <c:v>41.5</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>35.01</c:v>
+                  <c:v>34.74</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>35.27</c:v>
+                  <c:v>34.88</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>46.39</c:v>
+                  <c:v>47.09</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>39.19</c:v>
+                  <c:v>37.08</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>33.62</c:v>
+                  <c:v>34.3</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>16.99</c:v>
+                  <c:v>17.43</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>30.46</c:v>
+                  <c:v>30.18</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>28.24</c:v>
+                  <c:v>29.37</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1655,76 +1658,76 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>70.13</c:v>
+                  <c:v>68.64</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>61.25</c:v>
+                  <c:v>60.11</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>60.67</c:v>
+                  <c:v>60.26</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>58.17</c:v>
+                  <c:v>57.42</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>61.19</c:v>
+                  <c:v>60.1</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50.64</c:v>
+                  <c:v>50.29</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>57.66</c:v>
+                  <c:v>58.2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>49.17</c:v>
+                  <c:v>48.71</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>59.6</c:v>
+                  <c:v>61.2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>59.94</c:v>
+                  <c:v>60.1</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>59.4</c:v>
+                  <c:v>58.91</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>52.52</c:v>
+                  <c:v>51.78</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>51.18</c:v>
+                  <c:v>50.45</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>56.35</c:v>
+                  <c:v>55.45</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>54.24</c:v>
+                  <c:v>52.65</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>54.26</c:v>
+                  <c:v>53.91</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>52.02</c:v>
+                  <c:v>51.43</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>51.81</c:v>
+                  <c:v>51.17</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>55.42</c:v>
+                  <c:v>55.14</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>52.94</c:v>
+                  <c:v>51.72</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>50.94</c:v>
+                  <c:v>50.6</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>45.07</c:v>
+                  <c:v>44.66</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>48.55</c:v>
+                  <c:v>47.92</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>47.32</c:v>
+                  <c:v>47.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2781,22 +2784,22 @@
                   <c:v>113.1694952691261</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>114.9674982918469</c:v>
+                  <c:v>113.768829610033</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>122.1266180758187</c:v>
+                  <c:v>116.1303221795618</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>124.8339528715453</c:v>
+                  <c:v>118.7047295203143</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>122.5254387051666</c:v>
+                  <c:v>116.5095611113177</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>123.8829218426343</c:v>
+                  <c:v>117.8003931722659</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>123.3545573612726</c:v>
+                  <c:v>117.2979708632269</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3633,7 +3636,7 @@
         <v>14.48</v>
       </c>
       <c r="F14" s="11">
-        <v>0.3060016906170752</v>
+        <v>0.3067796610169491</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>25</v>
@@ -3647,13 +3650,13 @@
         <v>0.2</v>
       </c>
       <c r="D15" s="10">
-        <v>37.19</v>
+        <v>36.4</v>
       </c>
       <c r="E15" s="10">
-        <v>7.44</v>
+        <v>7.28</v>
       </c>
       <c r="F15" s="11">
-        <v>0.1572273879966188</v>
+        <v>0.1542372881355932</v>
       </c>
       <c r="G15" s="13" t="s">
         <v>27</v>
@@ -3673,7 +3676,7 @@
         <v>8.57</v>
       </c>
       <c r="F16" s="11">
-        <v>0.1811073541842773</v>
+        <v>0.1815677966101695</v>
       </c>
       <c r="G16" s="13" t="s">
         <v>27</v>
@@ -3693,7 +3696,7 @@
         <v>8.24</v>
       </c>
       <c r="F17" s="11">
-        <v>0.1741335587489434</v>
+        <v>0.1745762711864407</v>
       </c>
       <c r="G17" s="12" t="s">
         <v>25</v>
@@ -3713,7 +3716,7 @@
         <v>2.59</v>
       </c>
       <c r="F18" s="11">
-        <v>0.05473372781065088</v>
+        <v>0.0548728813559322</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>27</v>
@@ -3727,13 +3730,13 @@
         <v>0.1</v>
       </c>
       <c r="D19" s="10">
-        <v>59.97</v>
+        <v>60.43</v>
       </c>
       <c r="E19" s="10">
-        <v>6</v>
+        <v>6.04</v>
       </c>
       <c r="F19" s="11">
-        <v>0.1267962806424345</v>
+        <v>0.1279661016949152</v>
       </c>
       <c r="G19" s="12" t="s">
         <v>25</v>
@@ -3748,7 +3751,7 @@
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="10">
-        <v>47.32</v>
+        <v>47.2</v>
       </c>
       <c r="F20" s="11">
         <v>1</v>
@@ -3865,13 +3868,13 @@
         <v>45</v>
       </c>
       <c r="C6" s="10">
-        <v>70.13</v>
+        <v>68.64</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>46</v>
       </c>
       <c r="E6" s="10">
-        <v>70.13</v>
+        <v>68.64</v>
       </c>
       <c r="F6" s="14" t="s">
         <v>46</v>
@@ -3886,7 +3889,7 @@
         <v>20.63</v>
       </c>
       <c r="J6" s="10">
-        <v>12.64</v>
+        <v>11.18</v>
       </c>
       <c r="K6" s="10">
         <v>12.5</v>
@@ -3898,7 +3901,7 @@
         <v>8.52</v>
       </c>
       <c r="N6" s="10">
-        <v>7.8</v>
+        <v>7.77</v>
       </c>
       <c r="O6" s="10">
         <v>1191.44</v>
@@ -3915,13 +3918,13 @@
         <v>50</v>
       </c>
       <c r="C7" s="10">
-        <v>61.25</v>
+        <v>60.11</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E7" s="10">
-        <v>61.25</v>
+        <v>60.11</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>47</v>
@@ -3936,7 +3939,7 @@
         <v>18.11</v>
       </c>
       <c r="J7" s="10">
-        <v>11.06</v>
+        <v>9.06</v>
       </c>
       <c r="K7" s="10">
         <v>12.32</v>
@@ -3948,7 +3951,7 @@
         <v>3.89</v>
       </c>
       <c r="N7" s="10">
-        <v>7.41</v>
+        <v>8.27</v>
       </c>
       <c r="O7" s="10">
         <v>1408.55</v>
@@ -3965,13 +3968,13 @@
         <v>51</v>
       </c>
       <c r="C8" s="10">
-        <v>60.67</v>
+        <v>60.26</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="10">
-        <v>60.67</v>
+        <v>60.26</v>
       </c>
       <c r="F8" s="14" t="s">
         <v>47</v>
@@ -3986,7 +3989,7 @@
         <v>18.1</v>
       </c>
       <c r="J8" s="10">
-        <v>11.69</v>
+        <v>11.36</v>
       </c>
       <c r="K8" s="10">
         <v>12.48</v>
@@ -3998,7 +4001,7 @@
         <v>3.25</v>
       </c>
       <c r="N8" s="10">
-        <v>5.86</v>
+        <v>5.78</v>
       </c>
       <c r="O8" s="10">
         <v>1342.06</v>
@@ -4015,13 +4018,13 @@
         <v>52</v>
       </c>
       <c r="C9" s="10">
-        <v>58.17</v>
+        <v>57.42</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E9" s="10">
-        <v>58.17</v>
+        <v>57.42</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>47</v>
@@ -4036,7 +4039,7 @@
         <v>18.55</v>
       </c>
       <c r="J9" s="10">
-        <v>11.9</v>
+        <v>11.93</v>
       </c>
       <c r="K9" s="10">
         <v>11.76</v>
@@ -4048,7 +4051,7 @@
         <v>3.04</v>
       </c>
       <c r="N9" s="10">
-        <v>4.98</v>
+        <v>4.2</v>
       </c>
       <c r="O9" s="10">
         <v>1498.28</v>
@@ -4065,13 +4068,13 @@
         <v>53</v>
       </c>
       <c r="C10" s="10">
-        <v>61.19</v>
+        <v>60.1</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E10" s="10">
-        <v>46.08</v>
+        <v>45.35</v>
       </c>
       <c r="F10" s="14" t="s">
         <v>33</v>
@@ -4086,7 +4089,7 @@
         <v>18.62</v>
       </c>
       <c r="J10" s="10">
-        <v>12.85</v>
+        <v>12.6</v>
       </c>
       <c r="K10" s="10">
         <v>6.81</v>
@@ -4098,7 +4101,7 @@
         <v>7.91</v>
       </c>
       <c r="N10" s="10">
-        <v>6.96</v>
+        <v>6.12</v>
       </c>
       <c r="O10" s="10">
         <v>1492.15</v>
@@ -4115,13 +4118,13 @@
         <v>55</v>
       </c>
       <c r="C11" s="10">
-        <v>50.64</v>
+        <v>50.29</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E11" s="10">
-        <v>11.75</v>
+        <v>11.29</v>
       </c>
       <c r="F11" s="14" t="s">
         <v>56</v>
@@ -4130,13 +4133,13 @@
         <v>10</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I11" s="10">
         <v>17.21</v>
       </c>
       <c r="J11" s="10">
-        <v>11.22</v>
+        <v>11</v>
       </c>
       <c r="K11" s="10">
         <v>7.13</v>
@@ -4148,7 +4151,7 @@
         <v>2.68</v>
       </c>
       <c r="N11" s="10">
-        <v>4.69</v>
+        <v>4.56</v>
       </c>
       <c r="O11" s="10">
         <v>1197.6</v>
@@ -4165,13 +4168,13 @@
         <v>57</v>
       </c>
       <c r="C12" s="10">
-        <v>57.66</v>
+        <v>58.2</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E12" s="10">
-        <v>43.58</v>
+        <v>46.77</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>33</v>
@@ -4186,7 +4189,7 @@
         <v>16.1</v>
       </c>
       <c r="J12" s="10">
-        <v>11.23</v>
+        <v>11.33</v>
       </c>
       <c r="K12" s="10">
         <v>10.48</v>
@@ -4198,7 +4201,7 @@
         <v>7.08</v>
       </c>
       <c r="N12" s="10">
-        <v>3.99</v>
+        <v>4.43</v>
       </c>
       <c r="O12" s="10">
         <v>1132.11</v>
@@ -4215,13 +4218,13 @@
         <v>59</v>
       </c>
       <c r="C13" s="10">
-        <v>49.17</v>
+        <v>48.71</v>
       </c>
       <c r="D13" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E13" s="10">
-        <v>22.14</v>
+        <v>20.65</v>
       </c>
       <c r="F13" s="14" t="s">
         <v>56</v>
@@ -4236,7 +4239,7 @@
         <v>10.57</v>
       </c>
       <c r="J13" s="10">
-        <v>10.07</v>
+        <v>10.14</v>
       </c>
       <c r="K13" s="10">
         <v>11.94</v>
@@ -4248,7 +4251,7 @@
         <v>3.67</v>
       </c>
       <c r="N13" s="10">
-        <v>4.7</v>
+        <v>4.17</v>
       </c>
       <c r="O13" s="10">
         <v>1007.09</v>
@@ -4265,19 +4268,19 @@
         <v>60</v>
       </c>
       <c r="C14" s="10">
-        <v>59.6</v>
+        <v>61.2</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E14" s="10">
-        <v>52.25</v>
+        <v>57.76</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>47</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="H14" s="14" t="s">
         <v>58</v>
@@ -4286,7 +4289,7 @@
         <v>13.72</v>
       </c>
       <c r="J14" s="10">
-        <v>10.41</v>
+        <v>11.48</v>
       </c>
       <c r="K14" s="10">
         <v>14.81</v>
@@ -4298,7 +4301,7 @@
         <v>6.7</v>
       </c>
       <c r="N14" s="10">
-        <v>5.65</v>
+        <v>6.18</v>
       </c>
       <c r="O14" s="10">
         <v>1064.64</v>
@@ -4312,16 +4315,16 @@
     </row>
     <row r="15" spans="2:17">
       <c r="B15" s="14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C15" s="10">
-        <v>59.94</v>
+        <v>60.1</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E15" s="10">
-        <v>52.96</v>
+        <v>54.48</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>47</v>
@@ -4336,7 +4339,7 @@
         <v>14.34</v>
       </c>
       <c r="J15" s="10">
-        <v>11.49</v>
+        <v>11.6</v>
       </c>
       <c r="K15" s="10">
         <v>14.67</v>
@@ -4348,7 +4351,7 @@
         <v>6.86</v>
       </c>
       <c r="N15" s="10">
-        <v>4.39</v>
+        <v>4.44</v>
       </c>
       <c r="O15" s="10">
         <v>1120.18</v>
@@ -4362,16 +4365,16 @@
     </row>
     <row r="16" spans="2:17">
       <c r="B16" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C16" s="10">
-        <v>59.4</v>
+        <v>58.91</v>
       </c>
       <c r="D16" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E16" s="10">
-        <v>51.43</v>
+        <v>51.08</v>
       </c>
       <c r="F16" s="14" t="s">
         <v>47</v>
@@ -4386,7 +4389,7 @@
         <v>13.1</v>
       </c>
       <c r="J16" s="10">
-        <v>11.45</v>
+        <v>11.18</v>
       </c>
       <c r="K16" s="10">
         <v>13.35</v>
@@ -4398,7 +4401,7 @@
         <v>6.77</v>
       </c>
       <c r="N16" s="10">
-        <v>6.36</v>
+        <v>6.14</v>
       </c>
       <c r="O16" s="10">
         <v>1154.15</v>
@@ -4412,16 +4415,16 @@
     </row>
     <row r="17" spans="2:17">
       <c r="B17" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C17" s="10">
-        <v>52.52</v>
+        <v>51.78</v>
       </c>
       <c r="D17" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E17" s="10">
-        <v>32.74</v>
+        <v>31.03</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>56</v>
@@ -4436,7 +4439,7 @@
         <v>14.28</v>
       </c>
       <c r="J17" s="10">
-        <v>9.630000000000001</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="K17" s="10">
         <v>11.02</v>
@@ -4448,7 +4451,7 @@
         <v>3.36</v>
       </c>
       <c r="N17" s="10">
-        <v>6</v>
+        <v>5.42</v>
       </c>
       <c r="O17" s="10">
         <v>1129.93</v>
@@ -4462,16 +4465,16 @@
     </row>
     <row r="18" spans="2:17">
       <c r="B18" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C18" s="10">
-        <v>51.18</v>
+        <v>50.45</v>
       </c>
       <c r="D18" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E18" s="10">
-        <v>30.74</v>
+        <v>29.31</v>
       </c>
       <c r="F18" s="14" t="s">
         <v>56</v>
@@ -4498,7 +4501,7 @@
         <v>6.76</v>
       </c>
       <c r="N18" s="10">
-        <v>4.08</v>
+        <v>3.35</v>
       </c>
       <c r="O18" s="10">
         <v>1284.09</v>
@@ -4512,16 +4515,16 @@
     </row>
     <row r="19" spans="2:17">
       <c r="B19" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C19" s="10">
-        <v>56.35</v>
+        <v>55.45</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E19" s="10">
-        <v>46.17</v>
+        <v>44.81</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>33</v>
@@ -4530,13 +4533,13 @@
         <v>47</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="I19" s="10">
         <v>16.24</v>
       </c>
       <c r="J19" s="10">
-        <v>10.05</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="K19" s="10">
         <v>8.970000000000001</v>
@@ -4548,7 +4551,7 @@
         <v>6.96</v>
       </c>
       <c r="N19" s="10">
-        <v>5.92</v>
+        <v>5.19</v>
       </c>
       <c r="O19" s="10">
         <v>1245.32</v>
@@ -4562,16 +4565,16 @@
     </row>
     <row r="20" spans="2:17">
       <c r="B20" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C20" s="10">
-        <v>54.24</v>
+        <v>52.65</v>
       </c>
       <c r="D20" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E20" s="10">
-        <v>40.55</v>
+        <v>37.27</v>
       </c>
       <c r="F20" s="14" t="s">
         <v>33</v>
@@ -4586,7 +4589,7 @@
         <v>15.96</v>
       </c>
       <c r="J20" s="10">
-        <v>10.86</v>
+        <v>10.15</v>
       </c>
       <c r="K20" s="10">
         <v>7.16</v>
@@ -4598,7 +4601,7 @@
         <v>7.53</v>
       </c>
       <c r="N20" s="10">
-        <v>4.82</v>
+        <v>3.94</v>
       </c>
       <c r="O20" s="10">
         <v>1287.94</v>
@@ -4612,16 +4615,16 @@
     </row>
     <row r="21" spans="2:17">
       <c r="B21" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C21" s="10">
-        <v>54.26</v>
+        <v>53.91</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E21" s="10">
-        <v>41.03</v>
+        <v>41.5</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>33</v>
@@ -4636,7 +4639,7 @@
         <v>18.25</v>
       </c>
       <c r="J21" s="10">
-        <v>10.9</v>
+        <v>10.57</v>
       </c>
       <c r="K21" s="10">
         <v>8.119999999999999</v>
@@ -4648,7 +4651,7 @@
         <v>4.73</v>
       </c>
       <c r="N21" s="10">
-        <v>4.31</v>
+        <v>4.29</v>
       </c>
       <c r="O21" s="10">
         <v>1266.78</v>
@@ -4662,19 +4665,19 @@
     </row>
     <row r="22" spans="2:17">
       <c r="B22" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C22" s="10">
-        <v>52.02</v>
+        <v>51.43</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E22" s="10">
-        <v>35.01</v>
+        <v>34.74</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="G22" s="14" t="s">
         <v>47</v>
@@ -4686,7 +4689,7 @@
         <v>16.09</v>
       </c>
       <c r="J22" s="10">
-        <v>9.27</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="K22" s="10">
         <v>7.06</v>
@@ -4698,7 +4701,7 @@
         <v>7.01</v>
       </c>
       <c r="N22" s="10">
-        <v>4.67</v>
+        <v>4.71</v>
       </c>
       <c r="O22" s="10">
         <v>1306.86</v>
@@ -4712,19 +4715,19 @@
     </row>
     <row r="23" spans="2:17">
       <c r="B23" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C23" s="10">
-        <v>51.81</v>
+        <v>51.17</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E23" s="10">
-        <v>35.27</v>
+        <v>34.88</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="G23" s="14" t="s">
         <v>47</v>
@@ -4736,7 +4739,7 @@
         <v>16.07</v>
       </c>
       <c r="J23" s="10">
-        <v>10.69</v>
+        <v>10.07</v>
       </c>
       <c r="K23" s="10">
         <v>6.66</v>
@@ -4748,7 +4751,7 @@
         <v>4.67</v>
       </c>
       <c r="N23" s="10">
-        <v>5.73</v>
+        <v>5.71</v>
       </c>
       <c r="O23" s="10">
         <v>1376.07</v>
@@ -4762,16 +4765,16 @@
     </row>
     <row r="24" spans="2:17">
       <c r="B24" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C24" s="10">
-        <v>55.42</v>
+        <v>55.14</v>
       </c>
       <c r="D24" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="10">
-        <v>46.39</v>
+        <v>47.09</v>
       </c>
       <c r="F24" s="14" t="s">
         <v>33</v>
@@ -4786,7 +4789,7 @@
         <v>14.89</v>
       </c>
       <c r="J24" s="10">
-        <v>11.38</v>
+        <v>11.07</v>
       </c>
       <c r="K24" s="10">
         <v>6.78</v>
@@ -4798,7 +4801,7 @@
         <v>6.97</v>
       </c>
       <c r="N24" s="10">
-        <v>6.7</v>
+        <v>6.73</v>
       </c>
       <c r="O24" s="10">
         <v>1661.7</v>
@@ -4812,16 +4815,16 @@
     </row>
     <row r="25" spans="2:17">
       <c r="B25" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C25" s="10">
-        <v>52.94</v>
+        <v>51.72</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E25" s="10">
-        <v>39.19</v>
+        <v>37.08</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>33</v>
@@ -4836,7 +4839,7 @@
         <v>14.56</v>
       </c>
       <c r="J25" s="10">
-        <v>11.33</v>
+        <v>10.2</v>
       </c>
       <c r="K25" s="10">
         <v>4.79</v>
@@ -4848,7 +4851,7 @@
         <v>6.92</v>
       </c>
       <c r="N25" s="10">
-        <v>6.91</v>
+        <v>6.82</v>
       </c>
       <c r="O25" s="10">
         <v>1784.49</v>
@@ -4862,16 +4865,16 @@
     </row>
     <row r="26" spans="2:17">
       <c r="B26" s="14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C26" s="10">
-        <v>50.94</v>
+        <v>50.6</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E26" s="10">
-        <v>33.62</v>
+        <v>34.3</v>
       </c>
       <c r="F26" s="14" t="s">
         <v>56</v>
@@ -4886,7 +4889,7 @@
         <v>16.93</v>
       </c>
       <c r="J26" s="10">
-        <v>11.84</v>
+        <v>11.43</v>
       </c>
       <c r="K26" s="10">
         <v>4.7</v>
@@ -4898,7 +4901,7 @@
         <v>4.89</v>
       </c>
       <c r="N26" s="10">
-        <v>3.97</v>
+        <v>4.04</v>
       </c>
       <c r="O26" s="10">
         <v>1674.49</v>
@@ -4912,16 +4915,16 @@
     </row>
     <row r="27" spans="2:17">
       <c r="B27" s="14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C27" s="10">
-        <v>45.07</v>
+        <v>44.66</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E27" s="10">
-        <v>16.99</v>
+        <v>17.43</v>
       </c>
       <c r="F27" s="14" t="s">
         <v>56</v>
@@ -4936,7 +4939,7 @@
         <v>12.61</v>
       </c>
       <c r="J27" s="10">
-        <v>8.33</v>
+        <v>8.08</v>
       </c>
       <c r="K27" s="10">
         <v>2.48</v>
@@ -4948,7 +4951,7 @@
         <v>7</v>
       </c>
       <c r="N27" s="10">
-        <v>5.83</v>
+        <v>5.67</v>
       </c>
       <c r="O27" s="10">
         <v>1860.01</v>
@@ -4962,16 +4965,16 @@
     </row>
     <row r="28" spans="2:17">
       <c r="B28" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C28" s="10">
-        <v>48.55</v>
+        <v>47.92</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E28" s="10">
-        <v>30.46</v>
+        <v>30.18</v>
       </c>
       <c r="F28" s="14" t="s">
         <v>56</v>
@@ -4986,7 +4989,7 @@
         <v>15.32</v>
       </c>
       <c r="J28" s="10">
-        <v>8.99</v>
+        <v>8.35</v>
       </c>
       <c r="K28" s="10">
         <v>4.36</v>
@@ -4998,7 +5001,7 @@
         <v>6.86</v>
       </c>
       <c r="N28" s="10">
-        <v>4.41</v>
+        <v>4.42</v>
       </c>
       <c r="O28" s="10">
         <v>1780.68</v>
@@ -5012,16 +5015,16 @@
     </row>
     <row r="29" spans="2:17">
       <c r="B29" s="14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C29" s="10">
-        <v>47.32</v>
+        <v>47.2</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E29" s="10">
-        <v>28.24</v>
+        <v>29.37</v>
       </c>
       <c r="F29" s="14" t="s">
         <v>56</v>
@@ -5036,7 +5039,7 @@
         <v>14.48</v>
       </c>
       <c r="J29" s="10">
-        <v>7.44</v>
+        <v>7.28</v>
       </c>
       <c r="K29" s="10">
         <v>8.57</v>
@@ -5048,7 +5051,7 @@
         <v>2.59</v>
       </c>
       <c r="N29" s="10">
-        <v>6</v>
+        <v>6.04</v>
       </c>
       <c r="O29" s="14" t="s">
         <v>49</v>
@@ -5118,46 +5121,46 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C6" s="15">
         <v>-0.036358</v>
@@ -5166,27 +5169,27 @@
         <v>0.0278</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I6" s="14">
         <v>1</v>
       </c>
       <c r="J6" s="18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C7" s="15">
         <v>0.000137</v>
@@ -5195,27 +5198,27 @@
         <v>0.9441000000000001</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I7" s="14">
         <v>10</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C8" s="15">
         <v>-0.032628</v>
@@ -5224,27 +5227,27 @@
         <v>0.0592</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H8" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I8" s="14">
         <v>2</v>
       </c>
       <c r="J8" s="18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C9" s="15">
         <v>-0.002719</v>
@@ -5253,27 +5256,27 @@
         <v>0.7492</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I9" s="14">
         <v>7</v>
       </c>
       <c r="J9" s="18" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C10" s="15">
         <v>9.899999999999999E-05</v>
@@ -5282,27 +5285,27 @@
         <v>0.0223</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I10" s="14">
         <v>11</v>
       </c>
       <c r="J10" s="18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C11" s="15">
         <v>-8.000000000000001E-05</v>
@@ -5311,27 +5314,27 @@
         <v>0.2363</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I11" s="14">
         <v>12</v>
       </c>
       <c r="J11" s="18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C12" s="15">
         <v>-0.000221</v>
@@ -5340,27 +5343,27 @@
         <v>0.8799</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I12" s="14">
         <v>9</v>
       </c>
       <c r="J12" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C13" s="15">
         <v>-0.002852</v>
@@ -5369,27 +5372,27 @@
         <v>0.3781</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I13" s="14">
         <v>6</v>
       </c>
       <c r="J13" s="18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C14" s="15">
         <v>-0.029501</v>
@@ -5398,27 +5401,27 @@
         <v>0.0005999999999999999</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I14" s="14">
         <v>3</v>
       </c>
       <c r="J14" s="18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C15" s="15">
         <v>0.006628</v>
@@ -5427,27 +5430,27 @@
         <v>0.08939999999999999</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I15" s="14">
         <v>4</v>
       </c>
       <c r="J15" s="18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C16" s="15">
         <v>-0.005037</v>
@@ -5456,27 +5459,27 @@
         <v>0.2276</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I16" s="14">
         <v>5</v>
       </c>
       <c r="J16" s="18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C17" s="15">
         <v>-0.000575</v>
@@ -5485,40 +5488,40 @@
         <v>0.8627</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I17" s="14">
         <v>8</v>
       </c>
       <c r="J17" s="18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="39" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B39" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="40" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B40" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>45</v>
@@ -5548,57 +5551,57 @@
         <v>60</v>
       </c>
       <c r="L40" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M40" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N40" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O40" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P40" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q40" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R40" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="S40" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="T40" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U40" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="V40" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="W40" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="X40" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Y40" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Z40" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AA40" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="41" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B41" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C41" s="16">
         <v>0.050404</v>
@@ -5678,7 +5681,7 @@
     </row>
     <row r="42" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B42" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C42" s="16">
         <v>0.006803</v>
@@ -5758,7 +5761,7 @@
     </row>
     <row r="43" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B43" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C43" s="16">
         <v>0.033473</v>
@@ -5838,7 +5841,7 @@
     </row>
     <row r="44" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B44" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C44" s="16">
         <v>0.005801</v>
@@ -5918,7 +5921,7 @@
     </row>
     <row r="45" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B45" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C45" s="16">
         <v>0.000145</v>
@@ -5998,7 +6001,7 @@
     </row>
     <row r="46" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B46" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C46" s="16">
         <v>-6E-06</v>
@@ -6078,7 +6081,7 @@
     </row>
     <row r="47" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B47" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C47" s="16">
         <v>-0.00157</v>
@@ -6129,13 +6132,13 @@
         <v>3.8E-05</v>
       </c>
       <c r="S47" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="T47" s="16">
         <v>0.000618</v>
       </c>
       <c r="U47" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="V47" s="16">
         <v>0.000495</v>
@@ -6158,7 +6161,7 @@
     </row>
     <row r="48" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B48" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C48" s="16">
         <v>-0.013109</v>
@@ -6238,7 +6241,7 @@
     </row>
     <row r="49" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B49" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C49" s="16">
         <v>-0.045005</v>
@@ -6318,7 +6321,7 @@
     </row>
     <row r="50" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B50" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C50" s="16">
         <v>0.004475</v>
@@ -6398,7 +6401,7 @@
     </row>
     <row r="51" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B51" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C51" s="16">
         <v>-0.010339</v>
@@ -6478,10 +6481,10 @@
     </row>
     <row r="52" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B52" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D52" s="16">
         <v>0.023665</v>
@@ -6619,37 +6622,37 @@
   <sheetData>
     <row r="2" spans="2:7">
       <c r="B2" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="2:7">
       <c r="B3" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="2:7">
       <c r="B5" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="2:7">
       <c r="B6" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C6" s="16">
         <v>7.2336</v>
@@ -6658,18 +6661,18 @@
         <v>0.0072</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="2:7">
       <c r="B7" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C7" s="16">
         <v>0.5046</v>
@@ -6678,18 +6681,18 @@
         <v>0.4775</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="2:7">
       <c r="B8" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C8" s="16">
         <v>0.3229</v>
@@ -6698,18 +6701,18 @@
         <v>0.5699</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="2:7">
       <c r="B9" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C9" s="16">
         <v>0.2242</v>
@@ -6718,18 +6721,18 @@
         <v>0.6359</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="2:7">
       <c r="B10" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C10" s="16">
         <v>0.004</v>
@@ -6738,13 +6741,13 @@
         <v>0.9498</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -6776,36 +6779,36 @@
   <sheetData>
     <row r="2" spans="2:7">
       <c r="B2" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="2:7">
       <c r="B5" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="2:7">
       <c r="B6" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="2:7">
       <c r="B7" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="2:7">
       <c r="B8" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C8" s="16">
         <v>0.425</v>
@@ -6813,7 +6816,7 @@
     </row>
     <row r="9" spans="2:7">
       <c r="B9" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C9" s="16">
         <v>0.1599</v>
@@ -6821,7 +6824,7 @@
     </row>
     <row r="10" spans="2:7">
       <c r="B10" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C10" s="16">
         <v>0.3692</v>
@@ -6829,15 +6832,15 @@
     </row>
     <row r="11" spans="2:7">
       <c r="B11" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="2:7">
       <c r="B12" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C12" s="16">
         <v>0.5031</v>
@@ -6845,27 +6848,27 @@
     </row>
     <row r="14" spans="2:7">
       <c r="B14" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" spans="2:7">
       <c r="B15" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="2:7">
@@ -7030,18 +7033,18 @@
     </row>
     <row r="26" spans="2:7">
       <c r="B26" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="27" spans="2:7">
       <c r="B27" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="2:7">
@@ -7049,7 +7052,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D28" s="16">
         <v>0.02178040146827698</v>
@@ -7060,7 +7063,7 @@
         <v>2</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D29" s="16">
         <v>0.02076428011059761</v>
@@ -7071,7 +7074,7 @@
         <v>3</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D30" s="16">
         <v>0.01783575303852558</v>
@@ -7082,7 +7085,7 @@
         <v>4</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D31" s="16">
         <v>0.01772940717637539</v>
@@ -7093,7 +7096,7 @@
         <v>5</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D32" s="16">
         <v>0.01733604446053505</v>
@@ -7104,7 +7107,7 @@
         <v>6</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D33" s="16">
         <v>0.0167862419039011</v>
@@ -7115,7 +7118,7 @@
         <v>7</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D34" s="16">
         <v>0.01557330787181854</v>
@@ -7126,7 +7129,7 @@
         <v>8</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D35" s="16">
         <v>0.01539521757513285</v>
@@ -7137,7 +7140,7 @@
         <v>9</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D36" s="16">
         <v>0.01488733943551779</v>
@@ -7148,7 +7151,7 @@
         <v>10</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D37" s="16">
         <v>0.01360253803431988</v>
@@ -7159,7 +7162,7 @@
         <v>11</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D38" s="16">
         <v>0.0134799899533391</v>
@@ -7170,7 +7173,7 @@
         <v>12</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D39" s="16">
         <v>0.01324111688882113</v>
@@ -7181,7 +7184,7 @@
         <v>13</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D40" s="16">
         <v>0.01247525215148926</v>
@@ -7192,7 +7195,7 @@
         <v>14</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D41" s="16">
         <v>0.01242704410105944</v>
@@ -7203,7 +7206,7 @@
         <v>15</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D42" s="16">
         <v>0.01225554849952459</v>
@@ -7243,12 +7246,12 @@
   <sheetData>
     <row r="2" spans="2:7">
       <c r="B2" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="2:7">
       <c r="B3" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" spans="2:7">
@@ -7256,19 +7259,19 @@
         <v>18</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="2:7">
@@ -7279,16 +7282,16 @@
         <v>0.25</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F6" s="10">
         <v>60</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="2:7">
@@ -7299,16 +7302,16 @@
         <v>0.25</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F7" s="10">
         <v>50</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" spans="2:7">
@@ -7319,16 +7322,16 @@
         <v>0.25</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F8" s="10">
         <v>69</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="2:7">
@@ -7339,16 +7342,16 @@
         <v>0.25</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F9" s="10">
         <v>68</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="2:7">
@@ -7359,16 +7362,16 @@
         <v>0.25</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F10" s="10">
         <v>43</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="2:7">
@@ -7379,16 +7382,16 @@
         <v>0.2</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F11" s="10">
         <v>29</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="2:7">
@@ -7399,16 +7402,16 @@
         <v>0.2</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F12" s="10">
         <v>0</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="2:7">
@@ -7419,16 +7422,16 @@
         <v>0.2</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F13" s="10">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" spans="2:7">
@@ -7439,16 +7442,16 @@
         <v>0.2</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" spans="2:7">
@@ -7459,16 +7462,16 @@
         <v>0.2</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F15" s="10">
         <v>48</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="16" spans="2:7">
@@ -7479,16 +7482,16 @@
         <v>0.2</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F16" s="10">
         <v>56</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="17" spans="2:7">
@@ -7499,16 +7502,16 @@
         <v>0.2</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F17" s="10">
         <v>30</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18" spans="2:7">
@@ -7519,16 +7522,16 @@
         <v>0.2</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F18" s="10">
         <v>33</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="19" spans="2:7">
@@ -7539,16 +7542,16 @@
         <v>0.2</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F19" s="10">
         <v>80</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="20" spans="2:7">
@@ -7559,16 +7562,16 @@
         <v>0.2</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F20" s="10">
         <v>19</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="2:7">
@@ -7579,16 +7582,16 @@
         <v>0.15</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F21" s="10">
         <v>48</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="22" spans="2:7">
@@ -7599,16 +7602,16 @@
         <v>0.15</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F22" s="10">
         <v>53</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" spans="2:7">
@@ -7619,16 +7622,16 @@
         <v>0.15</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="24" spans="2:7">
@@ -7639,16 +7642,16 @@
         <v>0.15</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="25" spans="2:7">
@@ -7659,16 +7662,16 @@
         <v>0.1</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G25" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="26" spans="2:7">
@@ -7679,16 +7682,16 @@
         <v>0.1</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G26" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" spans="2:7">
@@ -7699,16 +7702,16 @@
         <v>0.1</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F27" s="10">
         <v>75</v>
       </c>
       <c r="G27" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28" spans="2:7">
@@ -7719,16 +7722,16 @@
         <v>0.1</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G28" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="2:7">
@@ -7739,16 +7742,16 @@
         <v>0.1</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F29" s="10">
         <v>38</v>
       </c>
       <c r="G29" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" spans="2:7">
@@ -7759,16 +7762,16 @@
         <v>0.1</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F30" s="10">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G30" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="31" spans="2:7">
@@ -7779,16 +7782,16 @@
         <v>0.1</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G31" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="32" spans="2:7">
@@ -7799,16 +7802,16 @@
         <v>0.1</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G32" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -7850,17 +7853,17 @@
   <sheetData>
     <row r="2" spans="2:3">
       <c r="B2" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="2:3">
       <c r="B3" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C5" s="14">
         <v>22</v>
@@ -7868,39 +7871,39 @@
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C6" s="16">
-        <v>0.1550909362864956</v>
+        <v>0.1483538183721982</v>
       </c>
     </row>
     <row r="7" spans="2:3">
       <c r="B7" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C7" s="16">
-        <v>0.1078486730660644</v>
+        <v>0.1067193675889328</v>
       </c>
     </row>
     <row r="8" spans="2:3">
       <c r="B8" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C8" s="16">
-        <v>0.0539510747016974</v>
+        <v>0.05631062061483348</v>
       </c>
     </row>
     <row r="9" spans="2:3">
       <c r="B9" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C9" s="16">
-        <v>-0.04912478825522304</v>
+        <v>0.0378424189052429</v>
       </c>
     </row>
     <row r="10" spans="2:3">
       <c r="B10" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C10" s="11">
         <v>0.5</v>
@@ -7908,7 +7911,7 @@
     </row>
     <row r="11" spans="2:3">
       <c r="B11" s="4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C11" s="11">
         <v>0.5454545454545454</v>
@@ -7916,15 +7919,15 @@
     </row>
     <row r="12" spans="2:3">
       <c r="B12" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C12" s="11">
-        <v>0.2335455736127263</v>
+        <v>0.1729797086322691</v>
       </c>
     </row>
     <row r="13" spans="2:3">
       <c r="B13" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C13" s="11">
         <v>0.306871980645762</v>
@@ -7932,7 +7935,7 @@
     </row>
     <row r="14" spans="2:3">
       <c r="B14" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C14" s="11">
         <v>0.4945612032498485</v>
@@ -7940,15 +7943,15 @@
     </row>
     <row r="15" spans="2:3">
       <c r="B15" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C15" s="10">
-        <v>0.5213441818233974</v>
+        <v>0.4192135232141344</v>
       </c>
     </row>
     <row r="16" spans="2:3">
       <c r="B16" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C16" s="10">
         <v>0.4775014136300051</v>
@@ -7956,24 +7959,24 @@
     </row>
     <row r="18" spans="2:12">
       <c r="B18" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="19" spans="2:12">
       <c r="B19" s="7" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="20" spans="2:12">
@@ -8015,16 +8018,16 @@
         <v>33</v>
       </c>
       <c r="C22" s="14">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D22" s="11">
-        <v>0.001598189831757129</v>
+        <v>-0.03516352497855219</v>
       </c>
       <c r="E22" s="11">
-        <v>0.03163927438071323</v>
+        <v>-0.01642933677034653</v>
       </c>
       <c r="F22" s="11">
-        <v>0.5555555555555556</v>
+        <v>0.4285714285714285</v>
       </c>
     </row>
     <row r="23" spans="2:12">
@@ -8032,21 +8035,21 @@
         <v>56</v>
       </c>
       <c r="C23" s="14">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D23" s="11">
-        <v>0.02947379187416812</v>
+        <v>0.05467139182258603</v>
       </c>
       <c r="E23" s="11">
-        <v>0.01347612765786038</v>
+        <v>0.05505192201341436</v>
       </c>
       <c r="F23" s="11">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="25" spans="2:12">
       <c r="B25" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="26" spans="2:12">
@@ -8054,34 +8057,34 @@
         <v>36</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>40</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="H26" s="7" t="s">
         <v>44</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27" spans="2:12">
@@ -8089,7 +8092,7 @@
         <v>45</v>
       </c>
       <c r="C27" s="10">
-        <v>70.13</v>
+        <v>68.64</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>46</v>
@@ -8098,7 +8101,7 @@
         <v>0.775</v>
       </c>
       <c r="F27" s="10">
-        <v>70.13</v>
+        <v>68.64</v>
       </c>
       <c r="G27" s="14" t="s">
         <v>46</v>
@@ -8110,7 +8113,7 @@
         <v>0.1412242748270999</v>
       </c>
       <c r="J27" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K27" s="10">
         <v>114.12242748271</v>
@@ -8124,7 +8127,7 @@
         <v>50</v>
       </c>
       <c r="C28" s="10">
-        <v>61.25</v>
+        <v>60.11</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>47</v>
@@ -8133,7 +8136,7 @@
         <v>0.5</v>
       </c>
       <c r="F28" s="10">
-        <v>61.25</v>
+        <v>60.11</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>47</v>
@@ -8145,7 +8148,7 @@
         <v>-0.02360228603883424</v>
       </c>
       <c r="J28" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K28" s="10">
         <v>111.4288773058169</v>
@@ -8159,7 +8162,7 @@
         <v>51</v>
       </c>
       <c r="C29" s="10">
-        <v>60.67</v>
+        <v>60.26</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>47</v>
@@ -8168,7 +8171,7 @@
         <v>0.5</v>
       </c>
       <c r="F29" s="10">
-        <v>60.67</v>
+        <v>60.26</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>47</v>
@@ -8180,7 +8183,7 @@
         <v>0.05820157071963994</v>
       </c>
       <c r="J29" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K29" s="10">
         <v>117.9142129885415</v>
@@ -8194,7 +8197,7 @@
         <v>52</v>
       </c>
       <c r="C30" s="10">
-        <v>58.17</v>
+        <v>57.42</v>
       </c>
       <c r="D30" s="14" t="s">
         <v>47</v>
@@ -8203,7 +8206,7 @@
         <v>0.5</v>
       </c>
       <c r="F30" s="10">
-        <v>58.17</v>
+        <v>57.42</v>
       </c>
       <c r="G30" s="14" t="s">
         <v>47</v>
@@ -8215,7 +8218,7 @@
         <v>-0.002045679045305226</v>
       </c>
       <c r="J30" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K30" s="10">
         <v>117.6729983538872</v>
@@ -8229,7 +8232,7 @@
         <v>53</v>
       </c>
       <c r="C31" s="10">
-        <v>46.08</v>
+        <v>45.35</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>33</v>
@@ -8238,7 +8241,7 @@
         <v>0.3</v>
       </c>
       <c r="F31" s="10">
-        <v>61.19</v>
+        <v>60.1</v>
       </c>
       <c r="G31" s="14" t="s">
         <v>47</v>
@@ -8250,7 +8253,7 @@
         <v>-0.05921991756860909</v>
       </c>
       <c r="J31" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K31" s="10">
         <v>110.7044130913189</v>
@@ -8264,7 +8267,7 @@
         <v>55</v>
       </c>
       <c r="C32" s="10">
-        <v>11.75</v>
+        <v>11.29</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>56</v>
@@ -8273,7 +8276,7 @@
         <v>0.1</v>
       </c>
       <c r="F32" s="10">
-        <v>50.64</v>
+        <v>50.29</v>
       </c>
       <c r="G32" s="14" t="s">
         <v>47</v>
@@ -8285,7 +8288,7 @@
         <v>-0.005468436873747495</v>
       </c>
       <c r="J32" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K32" s="10">
         <v>110.0990329966838</v>
@@ -8299,7 +8302,7 @@
         <v>57</v>
       </c>
       <c r="C33" s="10">
-        <v>43.58</v>
+        <v>46.77</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>33</v>
@@ -8308,7 +8311,7 @@
         <v>0.3</v>
       </c>
       <c r="F33" s="10">
-        <v>57.66</v>
+        <v>58.2</v>
       </c>
       <c r="G33" s="14" t="s">
         <v>47</v>
@@ -8320,7 +8323,7 @@
         <v>-0.03312928955666848</v>
       </c>
       <c r="J33" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K33" s="10">
         <v>106.4515302526274</v>
@@ -8334,7 +8337,7 @@
         <v>59</v>
       </c>
       <c r="C34" s="10">
-        <v>22.14</v>
+        <v>20.65</v>
       </c>
       <c r="D34" s="14" t="s">
         <v>56</v>
@@ -8343,7 +8346,7 @@
         <v>0.1</v>
       </c>
       <c r="F34" s="10">
-        <v>49.17</v>
+        <v>48.71</v>
       </c>
       <c r="G34" s="14" t="s">
         <v>33</v>
@@ -8355,7 +8358,7 @@
         <v>0.005714484306268553</v>
       </c>
       <c r="J34" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K34" s="10">
         <v>107.0598458516343</v>
@@ -8369,7 +8372,7 @@
         <v>60</v>
       </c>
       <c r="C35" s="10">
-        <v>52.25</v>
+        <v>57.76</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>47</v>
@@ -8378,7 +8381,7 @@
         <v>0.5</v>
       </c>
       <c r="F35" s="10">
-        <v>59.6</v>
+        <v>61.2</v>
       </c>
       <c r="G35" s="14" t="s">
         <v>47</v>
@@ -8390,7 +8393,7 @@
         <v>0.02608393447550339</v>
       </c>
       <c r="J35" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K35" s="10">
         <v>109.8523878557859</v>
@@ -8401,10 +8404,10 @@
     </row>
     <row r="36" spans="2:12">
       <c r="B36" s="14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C36" s="10">
-        <v>52.96</v>
+        <v>54.48</v>
       </c>
       <c r="D36" s="14" t="s">
         <v>47</v>
@@ -8413,7 +8416,7 @@
         <v>0.5</v>
       </c>
       <c r="F36" s="10">
-        <v>59.94</v>
+        <v>60.1</v>
       </c>
       <c r="G36" s="14" t="s">
         <v>47</v>
@@ -8425,7 +8428,7 @@
         <v>0.01516274170222642</v>
       </c>
       <c r="J36" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K36" s="10">
         <v>111.518051238216</v>
@@ -8436,10 +8439,10 @@
     </row>
     <row r="37" spans="2:12">
       <c r="B37" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C37" s="10">
-        <v>51.43</v>
+        <v>51.08</v>
       </c>
       <c r="D37" s="14" t="s">
         <v>47</v>
@@ -8448,7 +8451,7 @@
         <v>0.5</v>
       </c>
       <c r="F37" s="10">
-        <v>59.4</v>
+        <v>58.91</v>
       </c>
       <c r="G37" s="14" t="s">
         <v>47</v>
@@ -8460,7 +8463,7 @@
         <v>-0.0104925702898237</v>
       </c>
       <c r="J37" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K37" s="10">
         <v>110.3479402470148</v>
@@ -8471,10 +8474,10 @@
     </row>
     <row r="38" spans="2:12">
       <c r="B38" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C38" s="10">
-        <v>32.74</v>
+        <v>31.03</v>
       </c>
       <c r="D38" s="14" t="s">
         <v>56</v>
@@ -8483,7 +8486,7 @@
         <v>0.1</v>
       </c>
       <c r="F38" s="10">
-        <v>52.52</v>
+        <v>51.78</v>
       </c>
       <c r="G38" s="14" t="s">
         <v>47</v>
@@ -8495,7 +8498,7 @@
         <v>0.0136433230377103</v>
       </c>
       <c r="J38" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K38" s="10">
         <v>111.8534528423508</v>
@@ -8506,10 +8509,10 @@
     </row>
     <row r="39" spans="2:12">
       <c r="B39" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C39" s="10">
-        <v>30.74</v>
+        <v>29.31</v>
       </c>
       <c r="D39" s="14" t="s">
         <v>56</v>
@@ -8518,7 +8521,7 @@
         <v>0.1</v>
       </c>
       <c r="F39" s="10">
-        <v>51.18</v>
+        <v>50.45</v>
       </c>
       <c r="G39" s="14" t="s">
         <v>47</v>
@@ -8530,7 +8533,7 @@
         <v>-0.003019258774696476</v>
       </c>
       <c r="J39" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K39" s="10">
         <v>111.5157383233764</v>
@@ -8541,10 +8544,10 @@
     </row>
     <row r="40" spans="2:12">
       <c r="B40" s="14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C40" s="10">
-        <v>46.17</v>
+        <v>44.81</v>
       </c>
       <c r="D40" s="14" t="s">
         <v>33</v>
@@ -8553,7 +8556,7 @@
         <v>0.3</v>
       </c>
       <c r="F40" s="10">
-        <v>56.35</v>
+        <v>55.45</v>
       </c>
       <c r="G40" s="14" t="s">
         <v>47</v>
@@ -8565,7 +8568,7 @@
         <v>0.01026724054861401</v>
       </c>
       <c r="J40" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K40" s="10">
         <v>112.6606972336988</v>
@@ -8576,10 +8579,10 @@
     </row>
     <row r="41" spans="2:12">
       <c r="B41" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C41" s="10">
-        <v>40.55</v>
+        <v>37.27</v>
       </c>
       <c r="D41" s="14" t="s">
         <v>33</v>
@@ -8588,7 +8591,7 @@
         <v>0.3</v>
       </c>
       <c r="F41" s="10">
-        <v>54.24</v>
+        <v>52.65</v>
       </c>
       <c r="G41" s="14" t="s">
         <v>47</v>
@@ -8600,7 +8603,7 @@
         <v>-0.004928801031103957</v>
       </c>
       <c r="J41" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K41" s="10">
         <v>112.1054150730085</v>
@@ -8611,10 +8614,10 @@
     </row>
     <row r="42" spans="2:12">
       <c r="B42" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C42" s="10">
-        <v>41.03</v>
+        <v>41.5</v>
       </c>
       <c r="D42" s="14" t="s">
         <v>33</v>
@@ -8623,7 +8626,7 @@
         <v>0.3</v>
       </c>
       <c r="F42" s="10">
-        <v>54.26</v>
+        <v>53.91</v>
       </c>
       <c r="G42" s="14" t="s">
         <v>47</v>
@@ -8635,7 +8638,7 @@
         <v>0.00949178231421397</v>
       </c>
       <c r="J42" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K42" s="10">
         <v>113.1694952691261</v>
@@ -8646,19 +8649,19 @@
     </row>
     <row r="43" spans="2:12">
       <c r="B43" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C43" s="10">
-        <v>35.01</v>
+        <v>34.74</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="E43" s="9">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="F43" s="10">
-        <v>52.02</v>
+        <v>51.43</v>
       </c>
       <c r="G43" s="14" t="s">
         <v>47</v>
@@ -8667,13 +8670,13 @@
         <v>0.05295900096414319</v>
       </c>
       <c r="I43" s="11">
-        <v>0.01588770028924296</v>
+        <v>0.005295900096414319</v>
       </c>
       <c r="J43" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K43" s="10">
-        <v>114.9674982918469</v>
+        <v>113.768829610033</v>
       </c>
       <c r="L43" s="10">
         <v>115.4963741354999</v>
@@ -8681,19 +8684,19 @@
     </row>
     <row r="44" spans="2:12">
       <c r="B44" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C44" s="10">
-        <v>35.27</v>
+        <v>34.88</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="E44" s="9">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="F44" s="10">
-        <v>51.81</v>
+        <v>51.17</v>
       </c>
       <c r="G44" s="14" t="s">
         <v>47</v>
@@ -8702,13 +8705,13 @@
         <v>0.2075693823715363</v>
       </c>
       <c r="I44" s="11">
-        <v>0.0622708147114609</v>
+        <v>0.02075693823715363</v>
       </c>
       <c r="J44" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K44" s="10">
-        <v>122.1266180758187</v>
+        <v>116.1303221795618</v>
       </c>
       <c r="L44" s="10">
         <v>139.4698851809575</v>
@@ -8716,10 +8719,10 @@
     </row>
     <row r="45" spans="2:12">
       <c r="B45" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C45" s="10">
-        <v>46.39</v>
+        <v>47.09</v>
       </c>
       <c r="D45" s="14" t="s">
         <v>33</v>
@@ -8728,7 +8731,7 @@
         <v>0.3</v>
       </c>
       <c r="F45" s="10">
-        <v>55.42</v>
+        <v>55.14</v>
       </c>
       <c r="G45" s="14" t="s">
         <v>47</v>
@@ -8740,10 +8743,10 @@
         <v>0.0221682614190287</v>
       </c>
       <c r="J45" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K45" s="10">
-        <v>124.8339528715453</v>
+        <v>118.7047295203143</v>
       </c>
       <c r="L45" s="10">
         <v>149.7759014302021</v>
@@ -8751,10 +8754,10 @@
     </row>
     <row r="46" spans="2:12">
       <c r="B46" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C46" s="10">
-        <v>39.19</v>
+        <v>37.08</v>
       </c>
       <c r="D46" s="14" t="s">
         <v>33</v>
@@ -8763,7 +8766,7 @@
         <v>0.3</v>
       </c>
       <c r="F46" s="10">
-        <v>52.94</v>
+        <v>51.72</v>
       </c>
       <c r="G46" s="14" t="s">
         <v>47</v>
@@ -8775,10 +8778,10 @@
         <v>-0.01849267858043475</v>
       </c>
       <c r="J46" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K46" s="10">
-        <v>122.5254387051666</v>
+        <v>116.5095611113177</v>
       </c>
       <c r="L46" s="10">
         <v>140.5433760827234</v>
@@ -8786,10 +8789,10 @@
     </row>
     <row r="47" spans="2:12">
       <c r="B47" s="14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C47" s="10">
-        <v>33.62</v>
+        <v>34.3</v>
       </c>
       <c r="D47" s="14" t="s">
         <v>56</v>
@@ -8798,7 +8801,7 @@
         <v>0.1</v>
       </c>
       <c r="F47" s="10">
-        <v>50.94</v>
+        <v>50.6</v>
       </c>
       <c r="G47" s="14" t="s">
         <v>47</v>
@@ -8810,10 +8813,10 @@
         <v>0.01107919426213355</v>
       </c>
       <c r="J47" s="13" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K47" s="10">
-        <v>123.8829218426343</v>
+        <v>117.8003931722659</v>
       </c>
       <c r="L47" s="10">
         <v>156.1144497414892</v>
@@ -8821,10 +8824,10 @@
     </row>
     <row r="48" spans="2:12">
       <c r="B48" s="14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C48" s="10">
-        <v>16.99</v>
+        <v>17.43</v>
       </c>
       <c r="D48" s="14" t="s">
         <v>56</v>
@@ -8833,7 +8836,7 @@
         <v>0.1</v>
       </c>
       <c r="F48" s="10">
-        <v>45.07</v>
+        <v>44.66</v>
       </c>
       <c r="G48" s="14" t="s">
         <v>33</v>
@@ -8845,10 +8848,10 @@
         <v>-0.004265030833167561</v>
       </c>
       <c r="J48" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="K48" s="10">
-        <v>123.3545573612726</v>
+        <v>117.2979708632269</v>
       </c>
       <c r="L48" s="10">
         <v>149.4561203249849</v>
@@ -8856,7 +8859,7 @@
     </row>
     <row r="69" spans="2:2">
       <c r="B69" s="19" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -8882,7 +8885,7 @@
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" spans="2:5">
@@ -8943,104 +8946,104 @@
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="14" spans="2:5">
       <c r="B14" s="7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="14" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="17" spans="2:9">
       <c r="B17" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18" spans="2:9">
       <c r="B18" s="14" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="19" spans="2:9">
       <c r="B19" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="21" spans="2:9">
       <c r="B21" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="22" spans="2:9">
       <c r="B22" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D22" s="19"/>
       <c r="E22" s="19"/>
@@ -9051,10 +9054,10 @@
     </row>
     <row r="23" spans="2:9">
       <c r="B23" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D23" s="19"/>
       <c r="E23" s="19"/>
@@ -9065,10 +9068,10 @@
     </row>
     <row r="24" spans="2:9">
       <c r="B24" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D24" s="19"/>
       <c r="E24" s="19"/>
@@ -9079,10 +9082,10 @@
     </row>
     <row r="25" spans="2:9">
       <c r="B25" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D25" s="19"/>
       <c r="E25" s="19"/>
@@ -9093,10 +9096,10 @@
     </row>
     <row r="26" spans="2:9">
       <c r="B26" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D26" s="19"/>
       <c r="E26" s="19"/>
@@ -9107,10 +9110,10 @@
     </row>
     <row r="27" spans="2:9">
       <c r="B27" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D27" s="19"/>
       <c r="E27" s="19"/>
@@ -9121,10 +9124,10 @@
     </row>
     <row r="28" spans="2:9">
       <c r="B28" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D28" s="19"/>
       <c r="E28" s="19"/>
@@ -9135,10 +9138,10 @@
     </row>
     <row r="29" spans="2:9">
       <c r="B29" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D29" s="19"/>
       <c r="E29" s="19"/>
@@ -9149,10 +9152,10 @@
     </row>
     <row r="30" spans="2:9">
       <c r="B30" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D30" s="19"/>
       <c r="E30" s="19"/>

</xml_diff>

<commit_message>
test: enforce web and workbook score consistency
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
+++ b/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
@@ -24,15 +24,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="306">
   <si>
     <t>VN-INDEX QUARTERLY QUANT FACTOR WORKBOOK</t>
   </si>
   <si>
-    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-28 17:03:44  |  Source: output/exports/score_*.json</t>
-  </si>
-  <si>
-    <t>47.2</t>
+    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-29 15:03:12  |  Source: output/exports/score_*.json</t>
+  </si>
+  <si>
+    <t>47.7</t>
   </si>
   <si>
     <t>Raw Regime / Label</t>
@@ -44,7 +44,7 @@
     <t>CALIBRATED ACTION</t>
   </si>
   <si>
-    <t>🔴 SELL — 29.4</t>
+    <t>🔴 SELL — 34.0</t>
   </si>
   <si>
     <t>Recommended Equity</t>
@@ -62,7 +62,7 @@
     <t>Pillar Dispersion</t>
   </si>
   <si>
-    <t>MEDIUM (σ=13.67)</t>
+    <t>LOW (σ=13.67)</t>
   </si>
   <si>
     <t>Data As-Of</t>
@@ -188,15 +188,15 @@
     <t>2022-Q1</t>
   </si>
   <si>
+    <t>SELL</t>
+  </si>
+  <si>
     <t>HIGH</t>
   </si>
   <si>
     <t>2022-Q2</t>
   </si>
   <si>
-    <t>SELL</t>
-  </si>
-  <si>
     <t>2022-Q3</t>
   </si>
   <si>
@@ -695,13 +695,13 @@
     <t>model_quality</t>
   </si>
   <si>
-    <t>Accuracy=42.5% F1=0.369 → quality 40</t>
+    <t>Accuracy=42.5% F1=0.369</t>
   </si>
   <si>
     <t>ml_signal</t>
   </si>
   <si>
-    <t>Forecast: DOWN (conf=50%)</t>
+    <t>Forecast: DOWN (conf=50.0%)</t>
   </si>
   <si>
     <t>ftse_upgrade</t>
@@ -938,7 +938,7 @@
     <t>Data: vnstock (HOSE OHLCV, foreign flows, valuation), yfinance/FRED (DXY, US10Y, USD/JPY), SBV (rates, USD/VND), KBNN (VN yield curve).</t>
   </si>
   <si>
-    <t>Workbook generated at 2026-09-28 17:03:44 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
+    <t>Workbook generated at 2026-09-29 15:03:12 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
   </si>
   <si>
     <t>Disclaimer: for research purposes only. Not financial advice.</t>
@@ -1295,13 +1295,13 @@
                   <c:v>7.28</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.57</c:v>
+                  <c:v>8.08</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.24</c:v>
+                  <c:v>7.63</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.59</c:v>
+                  <c:v>4.16</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>6.04</c:v>
@@ -1479,76 +1479,76 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>68.64</c:v>
+                  <c:v>66.86</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>60.11</c:v>
+                  <c:v>62.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>60.26</c:v>
+                  <c:v>63.44</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>57.42</c:v>
+                  <c:v>60.22</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>45.35</c:v>
+                  <c:v>30.12</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>11.29</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>46.77</c:v>
+                  <c:v>40.99</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>20.65</c:v>
+                  <c:v>6.74</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>57.76</c:v>
+                  <c:v>50.08</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>54.48</c:v>
+                  <c:v>47.42</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>51.08</c:v>
+                  <c:v>45.78</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>31.03</c:v>
+                  <c:v>29.45</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>29.31</c:v>
+                  <c:v>23.54</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>44.81</c:v>
+                  <c:v>42.92</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>37.27</c:v>
+                  <c:v>33.65</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>41.5</c:v>
+                  <c:v>42.96</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>34.74</c:v>
+                  <c:v>34.51</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>34.88</c:v>
+                  <c:v>38.94</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>47.09</c:v>
+                  <c:v>49.86</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>37.08</c:v>
+                  <c:v>41.55</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>34.3</c:v>
+                  <c:v>40.48</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>17.43</c:v>
+                  <c:v>21.85</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>30.18</c:v>
+                  <c:v>30.12</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>29.37</c:v>
+                  <c:v>33.97</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1658,76 +1658,76 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>68.64</c:v>
+                  <c:v>66.86</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>60.11</c:v>
+                  <c:v>62.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>60.26</c:v>
+                  <c:v>63.44</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>57.42</c:v>
+                  <c:v>60.22</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>60.1</c:v>
+                  <c:v>59.69</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50.29</c:v>
+                  <c:v>51.25</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>58.2</c:v>
+                  <c:v>57.52</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>48.71</c:v>
+                  <c:v>45.88</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>61.2</c:v>
+                  <c:v>58.49</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>60.1</c:v>
+                  <c:v>57.35</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>58.91</c:v>
+                  <c:v>56.64</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>51.78</c:v>
+                  <c:v>50.28</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>50.45</c:v>
+                  <c:v>47.02</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>55.45</c:v>
+                  <c:v>53.7</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>52.65</c:v>
+                  <c:v>49.74</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>53.91</c:v>
+                  <c:v>53.13</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>51.43</c:v>
+                  <c:v>49.61</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>51.17</c:v>
+                  <c:v>51.03</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>55.14</c:v>
+                  <c:v>55.2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>51.72</c:v>
+                  <c:v>51.98</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>50.6</c:v>
+                  <c:v>51.47</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>44.66</c:v>
+                  <c:v>44.38</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>47.92</c:v>
+                  <c:v>46.59</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>47.2</c:v>
+                  <c:v>47.67</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2748,58 +2748,58 @@
                   <c:v>117.6729983538872</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>110.7044130913189</c:v>
+                  <c:v>115.3501365996978</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>110.0990329966838</c:v>
+                  <c:v>114.7193516593242</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>106.4515302526274</c:v>
+                  <c:v>110.9187810404491</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>107.0598458516343</c:v>
+                  <c:v>111.5526246739752</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>109.8523878557859</c:v>
+                  <c:v>114.4623560265416</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>111.518051238216</c:v>
+                  <c:v>115.5036939099769</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>110.3479402470148</c:v>
+                  <c:v>114.7765355337261</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>111.8534528423508</c:v>
+                  <c:v>116.3424688851619</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>111.5157383233764</c:v>
+                  <c:v>115.9912008651105</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>112.6606972336988</c:v>
+                  <c:v>117.1821104259152</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>112.1054150730085</c:v>
+                  <c:v>116.9895879903505</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>113.1694952691261</c:v>
+                  <c:v>118.1000276925845</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>113.768829610033</c:v>
+                  <c:v>118.7254736406282</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>116.1303221795618</c:v>
+                  <c:v>126.1186056112342</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>118.7047295203143</c:v>
+                  <c:v>128.9144358302274</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>116.5095611113177</c:v>
+                  <c:v>126.5304626040409</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>117.8003931722659</c:v>
+                  <c:v>130.7360293298443</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>117.2979708632269</c:v>
+                  <c:v>130.1784361337466</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3636,7 +3636,7 @@
         <v>14.48</v>
       </c>
       <c r="F14" s="11">
-        <v>0.3067796610169491</v>
+        <v>0.3037549821690791</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>25</v>
@@ -3656,7 +3656,7 @@
         <v>7.28</v>
       </c>
       <c r="F15" s="11">
-        <v>0.1542372881355932</v>
+        <v>0.1527165932452276</v>
       </c>
       <c r="G15" s="13" t="s">
         <v>27</v>
@@ -3670,13 +3670,13 @@
         <v>0.2</v>
       </c>
       <c r="D16" s="10">
-        <v>42.87</v>
+        <v>40.39</v>
       </c>
       <c r="E16" s="10">
-        <v>8.57</v>
+        <v>8.08</v>
       </c>
       <c r="F16" s="11">
-        <v>0.1815677966101695</v>
+        <v>0.1694986364589889</v>
       </c>
       <c r="G16" s="13" t="s">
         <v>27</v>
@@ -3690,13 +3690,13 @@
         <v>0.15</v>
       </c>
       <c r="D17" s="10">
-        <v>54.93</v>
+        <v>50.84</v>
       </c>
       <c r="E17" s="10">
-        <v>8.24</v>
+        <v>7.63</v>
       </c>
       <c r="F17" s="11">
-        <v>0.1745762711864407</v>
+        <v>0.1600587371512482</v>
       </c>
       <c r="G17" s="12" t="s">
         <v>25</v>
@@ -3710,13 +3710,13 @@
         <v>0.1</v>
       </c>
       <c r="D18" s="10">
-        <v>25.91</v>
+        <v>41.57</v>
       </c>
       <c r="E18" s="10">
-        <v>2.59</v>
+        <v>4.16</v>
       </c>
       <c r="F18" s="11">
-        <v>0.0548728813559322</v>
+        <v>0.08726662471155863</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>27</v>
@@ -3736,7 +3736,7 @@
         <v>6.04</v>
       </c>
       <c r="F19" s="11">
-        <v>0.1279661016949152</v>
+        <v>0.1267044262638976</v>
       </c>
       <c r="G19" s="12" t="s">
         <v>25</v>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="10">
-        <v>47.2</v>
+        <v>47.67</v>
       </c>
       <c r="F20" s="11">
         <v>1</v>
@@ -3868,13 +3868,13 @@
         <v>45</v>
       </c>
       <c r="C6" s="10">
-        <v>68.64</v>
+        <v>66.86</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>46</v>
       </c>
       <c r="E6" s="10">
-        <v>68.64</v>
+        <v>66.86</v>
       </c>
       <c r="F6" s="14" t="s">
         <v>46</v>
@@ -3895,10 +3895,10 @@
         <v>12.5</v>
       </c>
       <c r="L6" s="10">
-        <v>8.039999999999999</v>
+        <v>7.65</v>
       </c>
       <c r="M6" s="10">
-        <v>8.52</v>
+        <v>7.13</v>
       </c>
       <c r="N6" s="10">
         <v>7.77</v>
@@ -3918,13 +3918,13 @@
         <v>50</v>
       </c>
       <c r="C7" s="10">
-        <v>60.11</v>
+        <v>62.75</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E7" s="10">
-        <v>60.11</v>
+        <v>62.75</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>47</v>
@@ -3942,13 +3942,13 @@
         <v>9.06</v>
       </c>
       <c r="K7" s="10">
-        <v>12.32</v>
+        <v>12.3</v>
       </c>
       <c r="L7" s="10">
-        <v>8.460000000000001</v>
+        <v>11.28</v>
       </c>
       <c r="M7" s="10">
-        <v>3.89</v>
+        <v>3.73</v>
       </c>
       <c r="N7" s="10">
         <v>8.27</v>
@@ -3968,13 +3968,13 @@
         <v>51</v>
       </c>
       <c r="C8" s="10">
-        <v>60.26</v>
+        <v>63.44</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="10">
-        <v>60.26</v>
+        <v>63.44</v>
       </c>
       <c r="F8" s="14" t="s">
         <v>47</v>
@@ -3992,13 +3992,13 @@
         <v>11.36</v>
       </c>
       <c r="K8" s="10">
-        <v>12.48</v>
+        <v>12.5</v>
       </c>
       <c r="L8" s="10">
-        <v>9.289999999999999</v>
+        <v>11.75</v>
       </c>
       <c r="M8" s="10">
-        <v>3.25</v>
+        <v>3.95</v>
       </c>
       <c r="N8" s="10">
         <v>5.78</v>
@@ -4018,13 +4018,13 @@
         <v>52</v>
       </c>
       <c r="C9" s="10">
-        <v>57.42</v>
+        <v>60.22</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E9" s="10">
-        <v>57.42</v>
+        <v>60.22</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>47</v>
@@ -4042,13 +4042,13 @@
         <v>11.93</v>
       </c>
       <c r="K9" s="10">
-        <v>11.76</v>
+        <v>11.75</v>
       </c>
       <c r="L9" s="10">
-        <v>7.94</v>
+        <v>9.01</v>
       </c>
       <c r="M9" s="10">
-        <v>3.04</v>
+        <v>4.78</v>
       </c>
       <c r="N9" s="10">
         <v>4.2</v>
@@ -4068,22 +4068,22 @@
         <v>53</v>
       </c>
       <c r="C10" s="10">
-        <v>60.1</v>
+        <v>59.69</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E10" s="10">
-        <v>45.35</v>
+        <v>30.12</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>47</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I10" s="10">
         <v>18.62</v>
@@ -4092,13 +4092,13 @@
         <v>12.6</v>
       </c>
       <c r="K10" s="10">
-        <v>6.81</v>
+        <v>7.46</v>
       </c>
       <c r="L10" s="10">
-        <v>8.039999999999999</v>
+        <v>8.32</v>
       </c>
       <c r="M10" s="10">
-        <v>7.91</v>
+        <v>6.57</v>
       </c>
       <c r="N10" s="10">
         <v>6.12</v>
@@ -4115,19 +4115,19 @@
     </row>
     <row r="11" spans="2:17">
       <c r="B11" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C11" s="10">
-        <v>50.29</v>
+        <v>51.25</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E11" s="10">
-        <v>11.29</v>
+        <v>0</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>10</v>
@@ -4142,13 +4142,13 @@
         <v>11</v>
       </c>
       <c r="K11" s="10">
-        <v>7.13</v>
+        <v>7.34</v>
       </c>
       <c r="L11" s="10">
-        <v>7.71</v>
+        <v>7.1</v>
       </c>
       <c r="M11" s="10">
-        <v>2.68</v>
+        <v>4.04</v>
       </c>
       <c r="N11" s="10">
         <v>4.56</v>
@@ -4168,13 +4168,13 @@
         <v>57</v>
       </c>
       <c r="C12" s="10">
-        <v>58.2</v>
+        <v>57.52</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E12" s="10">
-        <v>46.77</v>
+        <v>40.99</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>33</v>
@@ -4192,13 +4192,13 @@
         <v>11.33</v>
       </c>
       <c r="K12" s="10">
-        <v>10.48</v>
+        <v>8.15</v>
       </c>
       <c r="L12" s="10">
-        <v>8.779999999999999</v>
+        <v>11.72</v>
       </c>
       <c r="M12" s="10">
-        <v>7.08</v>
+        <v>5.79</v>
       </c>
       <c r="N12" s="10">
         <v>4.43</v>
@@ -4218,16 +4218,16 @@
         <v>59</v>
       </c>
       <c r="C13" s="10">
-        <v>48.71</v>
+        <v>45.88</v>
       </c>
       <c r="D13" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E13" s="10">
-        <v>20.65</v>
+        <v>6.74</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>10</v>
@@ -4242,13 +4242,13 @@
         <v>10.14</v>
       </c>
       <c r="K13" s="10">
-        <v>11.94</v>
+        <v>10.06</v>
       </c>
       <c r="L13" s="10">
-        <v>8.220000000000001</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="M13" s="10">
-        <v>3.67</v>
+        <v>2.9</v>
       </c>
       <c r="N13" s="10">
         <v>4.17</v>
@@ -4268,13 +4268,13 @@
         <v>60</v>
       </c>
       <c r="C14" s="10">
-        <v>61.2</v>
+        <v>58.49</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E14" s="10">
-        <v>57.76</v>
+        <v>50.08</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>47</v>
@@ -4292,13 +4292,13 @@
         <v>11.48</v>
       </c>
       <c r="K14" s="10">
-        <v>14.81</v>
+        <v>12.87</v>
       </c>
       <c r="L14" s="10">
-        <v>8.31</v>
+        <v>8.85</v>
       </c>
       <c r="M14" s="10">
-        <v>6.7</v>
+        <v>5.39</v>
       </c>
       <c r="N14" s="10">
         <v>6.18</v>
@@ -4318,16 +4318,16 @@
         <v>62</v>
       </c>
       <c r="C15" s="10">
-        <v>60.1</v>
+        <v>57.35</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E15" s="10">
-        <v>54.48</v>
+        <v>47.42</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="G15" s="14" t="s">
         <v>47</v>
@@ -4342,13 +4342,13 @@
         <v>11.6</v>
       </c>
       <c r="K15" s="10">
-        <v>14.67</v>
+        <v>12.98</v>
       </c>
       <c r="L15" s="10">
-        <v>8.19</v>
+        <v>8.41</v>
       </c>
       <c r="M15" s="10">
-        <v>6.86</v>
+        <v>5.58</v>
       </c>
       <c r="N15" s="10">
         <v>4.44</v>
@@ -4368,16 +4368,16 @@
         <v>63</v>
       </c>
       <c r="C16" s="10">
-        <v>58.91</v>
+        <v>56.64</v>
       </c>
       <c r="D16" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E16" s="10">
-        <v>51.08</v>
+        <v>45.78</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="G16" s="14" t="s">
         <v>47</v>
@@ -4392,13 +4392,13 @@
         <v>11.18</v>
       </c>
       <c r="K16" s="10">
-        <v>13.35</v>
+        <v>11.95</v>
       </c>
       <c r="L16" s="10">
-        <v>8.369999999999999</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="M16" s="10">
-        <v>6.77</v>
+        <v>5.22</v>
       </c>
       <c r="N16" s="10">
         <v>6.14</v>
@@ -4418,16 +4418,16 @@
         <v>64</v>
       </c>
       <c r="C17" s="10">
-        <v>51.78</v>
+        <v>50.28</v>
       </c>
       <c r="D17" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E17" s="10">
-        <v>31.03</v>
+        <v>29.45</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G17" s="14" t="s">
         <v>10</v>
@@ -4442,13 +4442,13 @@
         <v>9.470000000000001</v>
       </c>
       <c r="K17" s="10">
-        <v>11.02</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="L17" s="10">
-        <v>8.23</v>
+        <v>8.52</v>
       </c>
       <c r="M17" s="10">
-        <v>3.36</v>
+        <v>3.06</v>
       </c>
       <c r="N17" s="10">
         <v>5.42</v>
@@ -4468,22 +4468,22 @@
         <v>65</v>
       </c>
       <c r="C18" s="10">
-        <v>50.45</v>
+        <v>47.02</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E18" s="10">
-        <v>29.31</v>
+        <v>23.54</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G18" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I18" s="10">
         <v>16.64</v>
@@ -4492,13 +4492,13 @@
         <v>4</v>
       </c>
       <c r="K18" s="10">
-        <v>11.64</v>
+        <v>10.56</v>
       </c>
       <c r="L18" s="10">
-        <v>8.06</v>
+        <v>7.28</v>
       </c>
       <c r="M18" s="10">
-        <v>6.76</v>
+        <v>5.19</v>
       </c>
       <c r="N18" s="10">
         <v>3.35</v>
@@ -4518,13 +4518,13 @@
         <v>66</v>
       </c>
       <c r="C19" s="10">
-        <v>55.45</v>
+        <v>53.7</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E19" s="10">
-        <v>44.81</v>
+        <v>42.92</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>33</v>
@@ -4542,13 +4542,13 @@
         <v>9.880000000000001</v>
       </c>
       <c r="K19" s="10">
-        <v>8.970000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="L19" s="10">
-        <v>8.210000000000001</v>
+        <v>8.09</v>
       </c>
       <c r="M19" s="10">
-        <v>6.96</v>
+        <v>5.7</v>
       </c>
       <c r="N19" s="10">
         <v>5.19</v>
@@ -4568,22 +4568,22 @@
         <v>67</v>
       </c>
       <c r="C20" s="10">
-        <v>52.65</v>
+        <v>49.74</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E20" s="10">
-        <v>37.27</v>
+        <v>33.65</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="G20" s="14" t="s">
         <v>47</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I20" s="10">
         <v>15.96</v>
@@ -4592,13 +4592,13 @@
         <v>10.15</v>
       </c>
       <c r="K20" s="10">
-        <v>7.16</v>
+        <v>7.12</v>
       </c>
       <c r="L20" s="10">
-        <v>7.91</v>
+        <v>6.38</v>
       </c>
       <c r="M20" s="10">
-        <v>7.53</v>
+        <v>6.19</v>
       </c>
       <c r="N20" s="10">
         <v>3.94</v>
@@ -4618,13 +4618,13 @@
         <v>68</v>
       </c>
       <c r="C21" s="10">
-        <v>53.91</v>
+        <v>53.13</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E21" s="10">
-        <v>41.5</v>
+        <v>42.96</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>33</v>
@@ -4642,10 +4642,10 @@
         <v>10.57</v>
       </c>
       <c r="K21" s="10">
-        <v>8.119999999999999</v>
+        <v>8.16</v>
       </c>
       <c r="L21" s="10">
-        <v>7.95</v>
+        <v>7.13</v>
       </c>
       <c r="M21" s="10">
         <v>4.73</v>
@@ -4668,16 +4668,16 @@
         <v>69</v>
       </c>
       <c r="C22" s="10">
-        <v>51.43</v>
+        <v>49.61</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E22" s="10">
-        <v>34.74</v>
+        <v>34.51</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G22" s="14" t="s">
         <v>47</v>
@@ -4692,13 +4692,13 @@
         <v>8.640000000000001</v>
       </c>
       <c r="K22" s="10">
-        <v>7.06</v>
+        <v>7.41</v>
       </c>
       <c r="L22" s="10">
-        <v>7.92</v>
+        <v>7.09</v>
       </c>
       <c r="M22" s="10">
-        <v>7.01</v>
+        <v>5.67</v>
       </c>
       <c r="N22" s="10">
         <v>4.71</v>
@@ -4718,16 +4718,16 @@
         <v>70</v>
       </c>
       <c r="C23" s="10">
-        <v>51.17</v>
+        <v>51.03</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E23" s="10">
-        <v>34.88</v>
+        <v>38.94</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="G23" s="14" t="s">
         <v>47</v>
@@ -4742,13 +4742,13 @@
         <v>10.07</v>
       </c>
       <c r="K23" s="10">
-        <v>6.66</v>
+        <v>7.1</v>
       </c>
       <c r="L23" s="10">
-        <v>7.99</v>
+        <v>7.46</v>
       </c>
       <c r="M23" s="10">
-        <v>4.67</v>
+        <v>4.62</v>
       </c>
       <c r="N23" s="10">
         <v>5.71</v>
@@ -4768,13 +4768,13 @@
         <v>71</v>
       </c>
       <c r="C24" s="10">
-        <v>55.14</v>
+        <v>55.2</v>
       </c>
       <c r="D24" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="10">
-        <v>47.09</v>
+        <v>49.86</v>
       </c>
       <c r="F24" s="14" t="s">
         <v>33</v>
@@ -4792,13 +4792,13 @@
         <v>11.07</v>
       </c>
       <c r="K24" s="10">
-        <v>6.78</v>
+        <v>7.47</v>
       </c>
       <c r="L24" s="10">
-        <v>8.699999999999999</v>
+        <v>9.34</v>
       </c>
       <c r="M24" s="10">
-        <v>6.97</v>
+        <v>5.7</v>
       </c>
       <c r="N24" s="10">
         <v>6.73</v>
@@ -4818,13 +4818,13 @@
         <v>72</v>
       </c>
       <c r="C25" s="10">
-        <v>51.72</v>
+        <v>51.98</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E25" s="10">
-        <v>37.08</v>
+        <v>41.55</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>33</v>
@@ -4833,7 +4833,7 @@
         <v>47</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I25" s="10">
         <v>14.56</v>
@@ -4842,13 +4842,13 @@
         <v>10.2</v>
       </c>
       <c r="K25" s="10">
-        <v>4.79</v>
+        <v>5.55</v>
       </c>
       <c r="L25" s="10">
-        <v>8.43</v>
+        <v>9.74</v>
       </c>
       <c r="M25" s="10">
-        <v>6.92</v>
+        <v>5.11</v>
       </c>
       <c r="N25" s="10">
         <v>6.82</v>
@@ -4868,22 +4868,22 @@
         <v>73</v>
       </c>
       <c r="C26" s="10">
-        <v>50.6</v>
+        <v>51.47</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E26" s="10">
-        <v>34.3</v>
+        <v>40.48</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="G26" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I26" s="10">
         <v>16.93</v>
@@ -4892,10 +4892,10 @@
         <v>11.43</v>
       </c>
       <c r="K26" s="10">
-        <v>4.7</v>
+        <v>5.79</v>
       </c>
       <c r="L26" s="10">
-        <v>8.609999999999999</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="M26" s="10">
         <v>4.89</v>
@@ -4918,22 +4918,22 @@
         <v>74</v>
       </c>
       <c r="C27" s="10">
-        <v>44.66</v>
+        <v>44.38</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E27" s="10">
-        <v>17.43</v>
+        <v>21.85</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G27" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I27" s="10">
         <v>12.61</v>
@@ -4942,13 +4942,13 @@
         <v>8.08</v>
       </c>
       <c r="K27" s="10">
-        <v>2.48</v>
+        <v>2.55</v>
       </c>
       <c r="L27" s="10">
-        <v>8.82</v>
+        <v>9.77</v>
       </c>
       <c r="M27" s="10">
-        <v>7</v>
+        <v>5.7</v>
       </c>
       <c r="N27" s="10">
         <v>5.67</v>
@@ -4968,22 +4968,22 @@
         <v>75</v>
       </c>
       <c r="C28" s="10">
-        <v>47.92</v>
+        <v>46.59</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E28" s="10">
-        <v>30.18</v>
+        <v>30.12</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I28" s="10">
         <v>15.32</v>
@@ -4992,13 +4992,13 @@
         <v>8.35</v>
       </c>
       <c r="K28" s="10">
-        <v>4.36</v>
+        <v>4.92</v>
       </c>
       <c r="L28" s="10">
-        <v>8.609999999999999</v>
+        <v>8.19</v>
       </c>
       <c r="M28" s="10">
-        <v>6.86</v>
+        <v>5.39</v>
       </c>
       <c r="N28" s="10">
         <v>4.42</v>
@@ -5018,16 +5018,16 @@
         <v>76</v>
       </c>
       <c r="C29" s="10">
-        <v>47.2</v>
+        <v>47.67</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E29" s="10">
-        <v>29.37</v>
+        <v>33.97</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>10</v>
@@ -5042,13 +5042,13 @@
         <v>7.28</v>
       </c>
       <c r="K29" s="10">
-        <v>8.57</v>
+        <v>8.08</v>
       </c>
       <c r="L29" s="10">
-        <v>8.24</v>
+        <v>7.63</v>
       </c>
       <c r="M29" s="10">
-        <v>2.59</v>
+        <v>4.16</v>
       </c>
       <c r="N29" s="10">
         <v>6.04</v>
@@ -5539,7 +5539,7 @@
         <v>53</v>
       </c>
       <c r="H40" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I40" s="7" t="s">
         <v>57</v>
@@ -7667,8 +7667,8 @@
       <c r="E25" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="F25" s="14" t="s">
-        <v>94</v>
+      <c r="F25" s="10">
+        <v>39.7</v>
       </c>
       <c r="G25" s="17" t="s">
         <v>187</v>
@@ -7687,8 +7687,8 @@
       <c r="E26" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="F26" s="14" t="s">
-        <v>94</v>
+      <c r="F26" s="10">
+        <v>42.5</v>
       </c>
       <c r="G26" s="17" t="s">
         <v>187</v>
@@ -7874,7 +7874,7 @@
         <v>241</v>
       </c>
       <c r="C6" s="16">
-        <v>0.1483538183721982</v>
+        <v>0.2837804645096819</v>
       </c>
     </row>
     <row r="7" spans="2:3">
@@ -7882,7 +7882,7 @@
         <v>242</v>
       </c>
       <c r="C7" s="16">
-        <v>0.1067193675889328</v>
+        <v>0.251270468661773</v>
       </c>
     </row>
     <row r="8" spans="2:3">
@@ -7890,7 +7890,7 @@
         <v>243</v>
       </c>
       <c r="C8" s="16">
-        <v>0.05631062061483348</v>
+        <v>0.03964834070416489</v>
       </c>
     </row>
     <row r="9" spans="2:3">
@@ -7898,7 +7898,7 @@
         <v>244</v>
       </c>
       <c r="C9" s="16">
-        <v>0.0378424189052429</v>
+        <v>-0.0254093732354602</v>
       </c>
     </row>
     <row r="10" spans="2:3">
@@ -7914,7 +7914,7 @@
         <v>246</v>
       </c>
       <c r="C11" s="11">
-        <v>0.5454545454545454</v>
+        <v>0.5909090909090909</v>
       </c>
     </row>
     <row r="12" spans="2:3">
@@ -7922,7 +7922,7 @@
         <v>247</v>
       </c>
       <c r="C12" s="11">
-        <v>0.1729797086322691</v>
+        <v>0.3017843613374662</v>
       </c>
     </row>
     <row r="13" spans="2:3">
@@ -7930,7 +7930,7 @@
         <v>248</v>
       </c>
       <c r="C13" s="11">
-        <v>0.306871980645762</v>
+        <v>0.3056281529812772</v>
       </c>
     </row>
     <row r="14" spans="2:3">
@@ -7946,7 +7946,7 @@
         <v>250</v>
       </c>
       <c r="C15" s="10">
-        <v>0.4192135232141344</v>
+        <v>0.6829570846962959</v>
       </c>
     </row>
     <row r="16" spans="2:3">
@@ -8001,13 +8001,13 @@
         <v>47</v>
       </c>
       <c r="C21" s="14">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D21" s="11">
-        <v>0.02110257050780219</v>
+        <v>0.02931877005550193</v>
       </c>
       <c r="E21" s="11">
-        <v>0.0131170626569212</v>
+        <v>0.02403825543019816</v>
       </c>
       <c r="F21" s="11">
         <v>0.5</v>
@@ -8018,33 +8018,33 @@
         <v>33</v>
       </c>
       <c r="C22" s="14">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D22" s="11">
-        <v>-0.03516352497855219</v>
+        <v>0.03282067277409505</v>
       </c>
       <c r="E22" s="11">
-        <v>-0.01642933677034653</v>
+        <v>0.03163927438071323</v>
       </c>
       <c r="F22" s="11">
-        <v>0.4285714285714285</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="23" spans="2:12">
       <c r="B23" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C23" s="14">
         <v>8</v>
       </c>
       <c r="D23" s="11">
-        <v>0.05467139182258603</v>
+        <v>-0.01185240655140339</v>
       </c>
       <c r="E23" s="11">
-        <v>0.05505192201341436</v>
+        <v>-0.02331096225865564</v>
       </c>
       <c r="F23" s="11">
-        <v>0.625</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="25" spans="2:12">
@@ -8092,7 +8092,7 @@
         <v>45</v>
       </c>
       <c r="C27" s="10">
-        <v>68.64</v>
+        <v>66.86</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>46</v>
@@ -8101,7 +8101,7 @@
         <v>0.775</v>
       </c>
       <c r="F27" s="10">
-        <v>68.64</v>
+        <v>66.86</v>
       </c>
       <c r="G27" s="14" t="s">
         <v>46</v>
@@ -8127,7 +8127,7 @@
         <v>50</v>
       </c>
       <c r="C28" s="10">
-        <v>60.11</v>
+        <v>62.75</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>47</v>
@@ -8136,7 +8136,7 @@
         <v>0.5</v>
       </c>
       <c r="F28" s="10">
-        <v>60.11</v>
+        <v>62.75</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>47</v>
@@ -8162,7 +8162,7 @@
         <v>51</v>
       </c>
       <c r="C29" s="10">
-        <v>60.26</v>
+        <v>63.44</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>47</v>
@@ -8171,7 +8171,7 @@
         <v>0.5</v>
       </c>
       <c r="F29" s="10">
-        <v>60.26</v>
+        <v>63.44</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>47</v>
@@ -8197,7 +8197,7 @@
         <v>52</v>
       </c>
       <c r="C30" s="10">
-        <v>57.42</v>
+        <v>60.22</v>
       </c>
       <c r="D30" s="14" t="s">
         <v>47</v>
@@ -8206,7 +8206,7 @@
         <v>0.5</v>
       </c>
       <c r="F30" s="10">
-        <v>57.42</v>
+        <v>60.22</v>
       </c>
       <c r="G30" s="14" t="s">
         <v>47</v>
@@ -8232,16 +8232,16 @@
         <v>53</v>
       </c>
       <c r="C31" s="10">
-        <v>45.35</v>
+        <v>30.12</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="E31" s="9">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="F31" s="10">
-        <v>60.1</v>
+        <v>59.69</v>
       </c>
       <c r="G31" s="14" t="s">
         <v>47</v>
@@ -8250,13 +8250,13 @@
         <v>-0.197399725228697</v>
       </c>
       <c r="I31" s="11">
-        <v>-0.05921991756860909</v>
+        <v>-0.0197399725228697</v>
       </c>
       <c r="J31" s="17" t="s">
         <v>267</v>
       </c>
       <c r="K31" s="10">
-        <v>110.7044130913189</v>
+        <v>115.3501365996978</v>
       </c>
       <c r="L31" s="10">
         <v>100.5170214194588</v>
@@ -8264,19 +8264,19 @@
     </row>
     <row r="32" spans="2:12">
       <c r="B32" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C32" s="10">
-        <v>11.29</v>
+        <v>0</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E32" s="9">
         <v>0.1</v>
       </c>
       <c r="F32" s="10">
-        <v>50.29</v>
+        <v>51.25</v>
       </c>
       <c r="G32" s="14" t="s">
         <v>47</v>
@@ -8291,7 +8291,7 @@
         <v>267</v>
       </c>
       <c r="K32" s="10">
-        <v>110.0990329966838</v>
+        <v>114.7193516593242</v>
       </c>
       <c r="L32" s="10">
         <v>95.02031155576445</v>
@@ -8302,7 +8302,7 @@
         <v>57</v>
       </c>
       <c r="C33" s="10">
-        <v>46.77</v>
+        <v>40.99</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>33</v>
@@ -8311,7 +8311,7 @@
         <v>0.3</v>
       </c>
       <c r="F33" s="10">
-        <v>58.2</v>
+        <v>57.52</v>
       </c>
       <c r="G33" s="14" t="s">
         <v>47</v>
@@ -8326,7 +8326,7 @@
         <v>267</v>
       </c>
       <c r="K33" s="10">
-        <v>106.4515302526274</v>
+        <v>110.9187810404491</v>
       </c>
       <c r="L33" s="10">
         <v>84.52712683811188</v>
@@ -8337,16 +8337,16 @@
         <v>59</v>
       </c>
       <c r="C34" s="10">
-        <v>20.65</v>
+        <v>6.74</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E34" s="9">
         <v>0.1</v>
       </c>
       <c r="F34" s="10">
-        <v>48.71</v>
+        <v>45.88</v>
       </c>
       <c r="G34" s="14" t="s">
         <v>33</v>
@@ -8361,7 +8361,7 @@
         <v>268</v>
       </c>
       <c r="K34" s="10">
-        <v>107.0598458516343</v>
+        <v>111.5526246739752</v>
       </c>
       <c r="L34" s="10">
         <v>89.35741623581549</v>
@@ -8372,7 +8372,7 @@
         <v>60</v>
       </c>
       <c r="C35" s="10">
-        <v>57.76</v>
+        <v>50.08</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>47</v>
@@ -8381,7 +8381,7 @@
         <v>0.5</v>
       </c>
       <c r="F35" s="10">
-        <v>61.2</v>
+        <v>58.49</v>
       </c>
       <c r="G35" s="14" t="s">
         <v>47</v>
@@ -8396,7 +8396,7 @@
         <v>267</v>
       </c>
       <c r="K35" s="10">
-        <v>109.8523878557859</v>
+        <v>114.4623560265416</v>
       </c>
       <c r="L35" s="10">
         <v>94.01900221580608</v>
@@ -8407,16 +8407,16 @@
         <v>62</v>
       </c>
       <c r="C36" s="10">
-        <v>54.48</v>
+        <v>47.42</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E36" s="9">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="F36" s="10">
-        <v>60.1</v>
+        <v>57.35</v>
       </c>
       <c r="G36" s="14" t="s">
         <v>47</v>
@@ -8425,13 +8425,13 @@
         <v>0.03032548340445285</v>
       </c>
       <c r="I36" s="11">
-        <v>0.01516274170222642</v>
-      </c>
-      <c r="J36" s="17" t="s">
-        <v>267</v>
+        <v>0.009097645021335853</v>
+      </c>
+      <c r="J36" s="13" t="s">
+        <v>268</v>
       </c>
       <c r="K36" s="10">
-        <v>111.518051238216</v>
+        <v>115.5036939099769</v>
       </c>
       <c r="L36" s="10">
         <v>96.87017390720473</v>
@@ -8442,16 +8442,16 @@
         <v>63</v>
       </c>
       <c r="C37" s="10">
-        <v>51.08</v>
+        <v>45.78</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E37" s="9">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="F37" s="10">
-        <v>58.91</v>
+        <v>56.64</v>
       </c>
       <c r="G37" s="14" t="s">
         <v>47</v>
@@ -8460,13 +8460,13 @@
         <v>-0.0209851405796474</v>
       </c>
       <c r="I37" s="11">
-        <v>-0.0104925702898237</v>
-      </c>
-      <c r="J37" s="13" t="s">
-        <v>268</v>
+        <v>-0.00629554217389422</v>
+      </c>
+      <c r="J37" s="17" t="s">
+        <v>267</v>
       </c>
       <c r="K37" s="10">
-        <v>110.3479402470148</v>
+        <v>114.7765355337261</v>
       </c>
       <c r="L37" s="10">
         <v>94.83733968978714</v>
@@ -8477,16 +8477,16 @@
         <v>64</v>
       </c>
       <c r="C38" s="10">
-        <v>31.03</v>
+        <v>29.45</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E38" s="9">
         <v>0.1</v>
       </c>
       <c r="F38" s="10">
-        <v>51.78</v>
+        <v>50.28</v>
       </c>
       <c r="G38" s="14" t="s">
         <v>47</v>
@@ -8501,7 +8501,7 @@
         <v>268</v>
       </c>
       <c r="K38" s="10">
-        <v>111.8534528423508</v>
+        <v>116.3424688851619</v>
       </c>
       <c r="L38" s="10">
         <v>107.7763043040354</v>
@@ -8512,19 +8512,19 @@
         <v>65</v>
       </c>
       <c r="C39" s="10">
-        <v>29.31</v>
+        <v>23.54</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E39" s="9">
         <v>0.1</v>
       </c>
       <c r="F39" s="10">
-        <v>50.45</v>
+        <v>47.02</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="H39" s="11">
         <v>-0.03019258774696476</v>
@@ -8536,7 +8536,7 @@
         <v>267</v>
       </c>
       <c r="K39" s="10">
-        <v>111.5157383233764</v>
+        <v>115.9912008651105</v>
       </c>
       <c r="L39" s="10">
         <v>104.5222587792923</v>
@@ -8547,7 +8547,7 @@
         <v>66</v>
       </c>
       <c r="C40" s="10">
-        <v>44.81</v>
+        <v>42.92</v>
       </c>
       <c r="D40" s="14" t="s">
         <v>33</v>
@@ -8556,7 +8556,7 @@
         <v>0.3</v>
       </c>
       <c r="F40" s="10">
-        <v>55.45</v>
+        <v>53.7</v>
       </c>
       <c r="G40" s="14" t="s">
         <v>47</v>
@@ -8571,7 +8571,7 @@
         <v>268</v>
       </c>
       <c r="K40" s="10">
-        <v>112.6606972336988</v>
+        <v>117.1821104259152</v>
       </c>
       <c r="L40" s="10">
         <v>108.0994426911972</v>
@@ -8582,31 +8582,31 @@
         <v>67</v>
       </c>
       <c r="C41" s="10">
-        <v>37.27</v>
+        <v>33.65</v>
       </c>
       <c r="D41" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E41" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="F41" s="10">
+        <v>49.74</v>
+      </c>
+      <c r="G41" s="14" t="s">
         <v>33</v>
-      </c>
-      <c r="E41" s="9">
-        <v>0.3</v>
-      </c>
-      <c r="F41" s="10">
-        <v>52.65</v>
-      </c>
-      <c r="G41" s="14" t="s">
-        <v>47</v>
       </c>
       <c r="H41" s="11">
         <v>-0.01642933677034653</v>
       </c>
       <c r="I41" s="11">
-        <v>-0.004928801031103957</v>
+        <v>-0.001642933677034653</v>
       </c>
       <c r="J41" s="17" t="s">
         <v>267</v>
       </c>
       <c r="K41" s="10">
-        <v>112.1054150730085</v>
+        <v>116.9895879903505</v>
       </c>
       <c r="L41" s="10">
         <v>106.3234405425367</v>
@@ -8617,7 +8617,7 @@
         <v>68</v>
       </c>
       <c r="C42" s="10">
-        <v>41.5</v>
+        <v>42.96</v>
       </c>
       <c r="D42" s="14" t="s">
         <v>33</v>
@@ -8626,7 +8626,7 @@
         <v>0.3</v>
       </c>
       <c r="F42" s="10">
-        <v>53.91</v>
+        <v>53.13</v>
       </c>
       <c r="G42" s="14" t="s">
         <v>47</v>
@@ -8641,7 +8641,7 @@
         <v>268</v>
       </c>
       <c r="K42" s="10">
-        <v>113.1694952691261</v>
+        <v>118.1000276925845</v>
       </c>
       <c r="L42" s="10">
         <v>109.6874370509635</v>
@@ -8652,19 +8652,19 @@
         <v>69</v>
       </c>
       <c r="C43" s="10">
-        <v>34.74</v>
+        <v>34.51</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E43" s="9">
         <v>0.1</v>
       </c>
       <c r="F43" s="10">
-        <v>51.43</v>
+        <v>49.61</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="H43" s="11">
         <v>0.05295900096414319</v>
@@ -8676,7 +8676,7 @@
         <v>268</v>
       </c>
       <c r="K43" s="10">
-        <v>113.768829610033</v>
+        <v>118.7254736406282</v>
       </c>
       <c r="L43" s="10">
         <v>115.4963741354999</v>
@@ -8687,16 +8687,16 @@
         <v>70</v>
       </c>
       <c r="C44" s="10">
-        <v>34.88</v>
+        <v>38.94</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E44" s="9">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="F44" s="10">
-        <v>51.17</v>
+        <v>51.03</v>
       </c>
       <c r="G44" s="14" t="s">
         <v>47</v>
@@ -8705,13 +8705,13 @@
         <v>0.2075693823715363</v>
       </c>
       <c r="I44" s="11">
-        <v>0.02075693823715363</v>
+        <v>0.0622708147114609</v>
       </c>
       <c r="J44" s="13" t="s">
         <v>268</v>
       </c>
       <c r="K44" s="10">
-        <v>116.1303221795618</v>
+        <v>126.1186056112342</v>
       </c>
       <c r="L44" s="10">
         <v>139.4698851809575</v>
@@ -8722,7 +8722,7 @@
         <v>71</v>
       </c>
       <c r="C45" s="10">
-        <v>47.09</v>
+        <v>49.86</v>
       </c>
       <c r="D45" s="14" t="s">
         <v>33</v>
@@ -8731,7 +8731,7 @@
         <v>0.3</v>
       </c>
       <c r="F45" s="10">
-        <v>55.14</v>
+        <v>55.2</v>
       </c>
       <c r="G45" s="14" t="s">
         <v>47</v>
@@ -8746,7 +8746,7 @@
         <v>268</v>
       </c>
       <c r="K45" s="10">
-        <v>118.7047295203143</v>
+        <v>128.9144358302274</v>
       </c>
       <c r="L45" s="10">
         <v>149.7759014302021</v>
@@ -8757,7 +8757,7 @@
         <v>72</v>
       </c>
       <c r="C46" s="10">
-        <v>37.08</v>
+        <v>41.55</v>
       </c>
       <c r="D46" s="14" t="s">
         <v>33</v>
@@ -8766,7 +8766,7 @@
         <v>0.3</v>
       </c>
       <c r="F46" s="10">
-        <v>51.72</v>
+        <v>51.98</v>
       </c>
       <c r="G46" s="14" t="s">
         <v>47</v>
@@ -8781,7 +8781,7 @@
         <v>267</v>
       </c>
       <c r="K46" s="10">
-        <v>116.5095611113177</v>
+        <v>126.5304626040409</v>
       </c>
       <c r="L46" s="10">
         <v>140.5433760827234</v>
@@ -8792,16 +8792,16 @@
         <v>73</v>
       </c>
       <c r="C47" s="10">
-        <v>34.3</v>
+        <v>40.48</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E47" s="9">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="F47" s="10">
-        <v>50.6</v>
+        <v>51.47</v>
       </c>
       <c r="G47" s="14" t="s">
         <v>47</v>
@@ -8810,13 +8810,13 @@
         <v>0.1107919426213355</v>
       </c>
       <c r="I47" s="11">
-        <v>0.01107919426213355</v>
+        <v>0.03323758278640065</v>
       </c>
       <c r="J47" s="13" t="s">
         <v>268</v>
       </c>
       <c r="K47" s="10">
-        <v>117.8003931722659</v>
+        <v>130.7360293298443</v>
       </c>
       <c r="L47" s="10">
         <v>156.1144497414892</v>
@@ -8827,16 +8827,16 @@
         <v>74</v>
       </c>
       <c r="C48" s="10">
-        <v>17.43</v>
+        <v>21.85</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E48" s="9">
         <v>0.1</v>
       </c>
       <c r="F48" s="10">
-        <v>44.66</v>
+        <v>44.38</v>
       </c>
       <c r="G48" s="14" t="s">
         <v>33</v>
@@ -8851,7 +8851,7 @@
         <v>267</v>
       </c>
       <c r="K48" s="10">
-        <v>117.2979708632269</v>
+        <v>130.1784361337466</v>
       </c>
       <c r="L48" s="10">
         <v>149.4561203249849</v>

</xml_diff>

<commit_message>
fix: reconcile PIT scoring, transparency, and generated artifacts
Merging after successful CI, workbook audit, and web/JSON consistency validation.
</commit_message>
<xml_diff>
--- a/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
+++ b/output/exports/VN_Index_Quant_Factor_Analysis.xlsx
@@ -24,15 +24,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="306">
   <si>
     <t>VN-INDEX QUARTERLY QUANT FACTOR WORKBOOK</t>
   </si>
   <si>
-    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-28 17:03:44  |  Source: output/exports/score_*.json</t>
-  </si>
-  <si>
-    <t>47.2</t>
+    <t>Latest full-model quarter: 2026-Q4  |  Generated at: 2026-09-29 15:03:12  |  Source: output/exports/score_*.json</t>
+  </si>
+  <si>
+    <t>47.7</t>
   </si>
   <si>
     <t>Raw Regime / Label</t>
@@ -44,7 +44,7 @@
     <t>CALIBRATED ACTION</t>
   </si>
   <si>
-    <t>🔴 SELL — 29.4</t>
+    <t>🔴 SELL — 34.0</t>
   </si>
   <si>
     <t>Recommended Equity</t>
@@ -62,7 +62,7 @@
     <t>Pillar Dispersion</t>
   </si>
   <si>
-    <t>MEDIUM (σ=13.67)</t>
+    <t>LOW (σ=13.67)</t>
   </si>
   <si>
     <t>Data As-Of</t>
@@ -188,15 +188,15 @@
     <t>2022-Q1</t>
   </si>
   <si>
+    <t>SELL</t>
+  </si>
+  <si>
     <t>HIGH</t>
   </si>
   <si>
     <t>2022-Q2</t>
   </si>
   <si>
-    <t>SELL</t>
-  </si>
-  <si>
     <t>2022-Q3</t>
   </si>
   <si>
@@ -695,13 +695,13 @@
     <t>model_quality</t>
   </si>
   <si>
-    <t>Accuracy=42.5% F1=0.369 → quality 40</t>
+    <t>Accuracy=42.5% F1=0.369</t>
   </si>
   <si>
     <t>ml_signal</t>
   </si>
   <si>
-    <t>Forecast: DOWN (conf=50%)</t>
+    <t>Forecast: DOWN (conf=50.0%)</t>
   </si>
   <si>
     <t>ftse_upgrade</t>
@@ -938,7 +938,7 @@
     <t>Data: vnstock (HOSE OHLCV, foreign flows, valuation), yfinance/FRED (DXY, US10Y, USD/JPY), SBV (rates, USD/VND), KBNN (VN yield curve).</t>
   </si>
   <si>
-    <t>Workbook generated at 2026-09-28 17:03:44 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
+    <t>Workbook generated at 2026-09-29 15:03:12 from output/exports/score_*.json, data/scores/quarterly_scores_history.parquet and data/scores/vnindex_quarterly_close.json.</t>
   </si>
   <si>
     <t>Disclaimer: for research purposes only. Not financial advice.</t>
@@ -1295,13 +1295,13 @@
                   <c:v>7.28</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.57</c:v>
+                  <c:v>8.08</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.24</c:v>
+                  <c:v>7.63</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.59</c:v>
+                  <c:v>4.16</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>6.04</c:v>
@@ -1479,76 +1479,76 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>68.64</c:v>
+                  <c:v>66.86</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>60.11</c:v>
+                  <c:v>62.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>60.26</c:v>
+                  <c:v>63.44</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>57.42</c:v>
+                  <c:v>60.22</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>45.35</c:v>
+                  <c:v>30.12</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>11.29</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>46.77</c:v>
+                  <c:v>40.99</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>20.65</c:v>
+                  <c:v>6.74</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>57.76</c:v>
+                  <c:v>50.08</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>54.48</c:v>
+                  <c:v>47.42</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>51.08</c:v>
+                  <c:v>45.78</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>31.03</c:v>
+                  <c:v>29.45</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>29.31</c:v>
+                  <c:v>23.54</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>44.81</c:v>
+                  <c:v>42.92</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>37.27</c:v>
+                  <c:v>33.65</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>41.5</c:v>
+                  <c:v>42.96</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>34.74</c:v>
+                  <c:v>34.51</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>34.88</c:v>
+                  <c:v>38.94</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>47.09</c:v>
+                  <c:v>49.86</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>37.08</c:v>
+                  <c:v>41.55</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>34.3</c:v>
+                  <c:v>40.48</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>17.43</c:v>
+                  <c:v>21.85</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>30.18</c:v>
+                  <c:v>30.12</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>29.37</c:v>
+                  <c:v>33.97</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1658,76 +1658,76 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="24"/>
                 <c:pt idx="0">
-                  <c:v>68.64</c:v>
+                  <c:v>66.86</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>60.11</c:v>
+                  <c:v>62.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>60.26</c:v>
+                  <c:v>63.44</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>57.42</c:v>
+                  <c:v>60.22</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>60.1</c:v>
+                  <c:v>59.69</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>50.29</c:v>
+                  <c:v>51.25</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>58.2</c:v>
+                  <c:v>57.52</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>48.71</c:v>
+                  <c:v>45.88</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>61.2</c:v>
+                  <c:v>58.49</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>60.1</c:v>
+                  <c:v>57.35</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>58.91</c:v>
+                  <c:v>56.64</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>51.78</c:v>
+                  <c:v>50.28</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>50.45</c:v>
+                  <c:v>47.02</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>55.45</c:v>
+                  <c:v>53.7</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>52.65</c:v>
+                  <c:v>49.74</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>53.91</c:v>
+                  <c:v>53.13</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>51.43</c:v>
+                  <c:v>49.61</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>51.17</c:v>
+                  <c:v>51.03</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>55.14</c:v>
+                  <c:v>55.2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>51.72</c:v>
+                  <c:v>51.98</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>50.6</c:v>
+                  <c:v>51.47</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>44.66</c:v>
+                  <c:v>44.38</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>47.92</c:v>
+                  <c:v>46.59</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>47.2</c:v>
+                  <c:v>47.67</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2748,58 +2748,58 @@
                   <c:v>117.6729983538872</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>110.7044130913189</c:v>
+                  <c:v>115.3501365996978</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>110.0990329966838</c:v>
+                  <c:v>114.7193516593242</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>106.4515302526274</c:v>
+                  <c:v>110.9187810404491</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>107.0598458516343</c:v>
+                  <c:v>111.5526246739752</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>109.8523878557859</c:v>
+                  <c:v>114.4623560265416</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>111.518051238216</c:v>
+                  <c:v>115.5036939099769</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>110.3479402470148</c:v>
+                  <c:v>114.7765355337261</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>111.8534528423508</c:v>
+                  <c:v>116.3424688851619</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>111.5157383233764</c:v>
+                  <c:v>115.9912008651105</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>112.6606972336988</c:v>
+                  <c:v>117.1821104259152</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>112.1054150730085</c:v>
+                  <c:v>116.9895879903505</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>113.1694952691261</c:v>
+                  <c:v>118.1000276925845</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>113.768829610033</c:v>
+                  <c:v>118.7254736406282</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>116.1303221795618</c:v>
+                  <c:v>126.1186056112342</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>118.7047295203143</c:v>
+                  <c:v>128.9144358302274</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>116.5095611113177</c:v>
+                  <c:v>126.5304626040409</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>117.8003931722659</c:v>
+                  <c:v>130.7360293298443</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>117.2979708632269</c:v>
+                  <c:v>130.1784361337466</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3636,7 +3636,7 @@
         <v>14.48</v>
       </c>
       <c r="F14" s="11">
-        <v>0.3067796610169491</v>
+        <v>0.3037549821690791</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>25</v>
@@ -3656,7 +3656,7 @@
         <v>7.28</v>
       </c>
       <c r="F15" s="11">
-        <v>0.1542372881355932</v>
+        <v>0.1527165932452276</v>
       </c>
       <c r="G15" s="13" t="s">
         <v>27</v>
@@ -3670,13 +3670,13 @@
         <v>0.2</v>
       </c>
       <c r="D16" s="10">
-        <v>42.87</v>
+        <v>40.39</v>
       </c>
       <c r="E16" s="10">
-        <v>8.57</v>
+        <v>8.08</v>
       </c>
       <c r="F16" s="11">
-        <v>0.1815677966101695</v>
+        <v>0.1694986364589889</v>
       </c>
       <c r="G16" s="13" t="s">
         <v>27</v>
@@ -3690,13 +3690,13 @@
         <v>0.15</v>
       </c>
       <c r="D17" s="10">
-        <v>54.93</v>
+        <v>50.84</v>
       </c>
       <c r="E17" s="10">
-        <v>8.24</v>
+        <v>7.63</v>
       </c>
       <c r="F17" s="11">
-        <v>0.1745762711864407</v>
+        <v>0.1600587371512482</v>
       </c>
       <c r="G17" s="12" t="s">
         <v>25</v>
@@ -3710,13 +3710,13 @@
         <v>0.1</v>
       </c>
       <c r="D18" s="10">
-        <v>25.91</v>
+        <v>41.57</v>
       </c>
       <c r="E18" s="10">
-        <v>2.59</v>
+        <v>4.16</v>
       </c>
       <c r="F18" s="11">
-        <v>0.0548728813559322</v>
+        <v>0.08726662471155863</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>27</v>
@@ -3736,7 +3736,7 @@
         <v>6.04</v>
       </c>
       <c r="F19" s="11">
-        <v>0.1279661016949152</v>
+        <v>0.1267044262638976</v>
       </c>
       <c r="G19" s="12" t="s">
         <v>25</v>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="10">
-        <v>47.2</v>
+        <v>47.67</v>
       </c>
       <c r="F20" s="11">
         <v>1</v>
@@ -3868,13 +3868,13 @@
         <v>45</v>
       </c>
       <c r="C6" s="10">
-        <v>68.64</v>
+        <v>66.86</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>46</v>
       </c>
       <c r="E6" s="10">
-        <v>68.64</v>
+        <v>66.86</v>
       </c>
       <c r="F6" s="14" t="s">
         <v>46</v>
@@ -3895,10 +3895,10 @@
         <v>12.5</v>
       </c>
       <c r="L6" s="10">
-        <v>8.039999999999999</v>
+        <v>7.65</v>
       </c>
       <c r="M6" s="10">
-        <v>8.52</v>
+        <v>7.13</v>
       </c>
       <c r="N6" s="10">
         <v>7.77</v>
@@ -3918,13 +3918,13 @@
         <v>50</v>
       </c>
       <c r="C7" s="10">
-        <v>60.11</v>
+        <v>62.75</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E7" s="10">
-        <v>60.11</v>
+        <v>62.75</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>47</v>
@@ -3942,13 +3942,13 @@
         <v>9.06</v>
       </c>
       <c r="K7" s="10">
-        <v>12.32</v>
+        <v>12.3</v>
       </c>
       <c r="L7" s="10">
-        <v>8.460000000000001</v>
+        <v>11.28</v>
       </c>
       <c r="M7" s="10">
-        <v>3.89</v>
+        <v>3.73</v>
       </c>
       <c r="N7" s="10">
         <v>8.27</v>
@@ -3968,13 +3968,13 @@
         <v>51</v>
       </c>
       <c r="C8" s="10">
-        <v>60.26</v>
+        <v>63.44</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="10">
-        <v>60.26</v>
+        <v>63.44</v>
       </c>
       <c r="F8" s="14" t="s">
         <v>47</v>
@@ -3992,13 +3992,13 @@
         <v>11.36</v>
       </c>
       <c r="K8" s="10">
-        <v>12.48</v>
+        <v>12.5</v>
       </c>
       <c r="L8" s="10">
-        <v>9.289999999999999</v>
+        <v>11.75</v>
       </c>
       <c r="M8" s="10">
-        <v>3.25</v>
+        <v>3.95</v>
       </c>
       <c r="N8" s="10">
         <v>5.78</v>
@@ -4018,13 +4018,13 @@
         <v>52</v>
       </c>
       <c r="C9" s="10">
-        <v>57.42</v>
+        <v>60.22</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E9" s="10">
-        <v>57.42</v>
+        <v>60.22</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>47</v>
@@ -4042,13 +4042,13 @@
         <v>11.93</v>
       </c>
       <c r="K9" s="10">
-        <v>11.76</v>
+        <v>11.75</v>
       </c>
       <c r="L9" s="10">
-        <v>7.94</v>
+        <v>9.01</v>
       </c>
       <c r="M9" s="10">
-        <v>3.04</v>
+        <v>4.78</v>
       </c>
       <c r="N9" s="10">
         <v>4.2</v>
@@ -4068,22 +4068,22 @@
         <v>53</v>
       </c>
       <c r="C10" s="10">
-        <v>60.1</v>
+        <v>59.69</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E10" s="10">
-        <v>45.35</v>
+        <v>30.12</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>47</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I10" s="10">
         <v>18.62</v>
@@ -4092,13 +4092,13 @@
         <v>12.6</v>
       </c>
       <c r="K10" s="10">
-        <v>6.81</v>
+        <v>7.46</v>
       </c>
       <c r="L10" s="10">
-        <v>8.039999999999999</v>
+        <v>8.32</v>
       </c>
       <c r="M10" s="10">
-        <v>7.91</v>
+        <v>6.57</v>
       </c>
       <c r="N10" s="10">
         <v>6.12</v>
@@ -4115,19 +4115,19 @@
     </row>
     <row r="11" spans="2:17">
       <c r="B11" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C11" s="10">
-        <v>50.29</v>
+        <v>51.25</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E11" s="10">
-        <v>11.29</v>
+        <v>0</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>10</v>
@@ -4142,13 +4142,13 @@
         <v>11</v>
       </c>
       <c r="K11" s="10">
-        <v>7.13</v>
+        <v>7.34</v>
       </c>
       <c r="L11" s="10">
-        <v>7.71</v>
+        <v>7.1</v>
       </c>
       <c r="M11" s="10">
-        <v>2.68</v>
+        <v>4.04</v>
       </c>
       <c r="N11" s="10">
         <v>4.56</v>
@@ -4168,13 +4168,13 @@
         <v>57</v>
       </c>
       <c r="C12" s="10">
-        <v>58.2</v>
+        <v>57.52</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E12" s="10">
-        <v>46.77</v>
+        <v>40.99</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>33</v>
@@ -4192,13 +4192,13 @@
         <v>11.33</v>
       </c>
       <c r="K12" s="10">
-        <v>10.48</v>
+        <v>8.15</v>
       </c>
       <c r="L12" s="10">
-        <v>8.779999999999999</v>
+        <v>11.72</v>
       </c>
       <c r="M12" s="10">
-        <v>7.08</v>
+        <v>5.79</v>
       </c>
       <c r="N12" s="10">
         <v>4.43</v>
@@ -4218,16 +4218,16 @@
         <v>59</v>
       </c>
       <c r="C13" s="10">
-        <v>48.71</v>
+        <v>45.88</v>
       </c>
       <c r="D13" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E13" s="10">
-        <v>20.65</v>
+        <v>6.74</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>10</v>
@@ -4242,13 +4242,13 @@
         <v>10.14</v>
       </c>
       <c r="K13" s="10">
-        <v>11.94</v>
+        <v>10.06</v>
       </c>
       <c r="L13" s="10">
-        <v>8.220000000000001</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="M13" s="10">
-        <v>3.67</v>
+        <v>2.9</v>
       </c>
       <c r="N13" s="10">
         <v>4.17</v>
@@ -4268,13 +4268,13 @@
         <v>60</v>
       </c>
       <c r="C14" s="10">
-        <v>61.2</v>
+        <v>58.49</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E14" s="10">
-        <v>57.76</v>
+        <v>50.08</v>
       </c>
       <c r="F14" s="14" t="s">
         <v>47</v>
@@ -4292,13 +4292,13 @@
         <v>11.48</v>
       </c>
       <c r="K14" s="10">
-        <v>14.81</v>
+        <v>12.87</v>
       </c>
       <c r="L14" s="10">
-        <v>8.31</v>
+        <v>8.85</v>
       </c>
       <c r="M14" s="10">
-        <v>6.7</v>
+        <v>5.39</v>
       </c>
       <c r="N14" s="10">
         <v>6.18</v>
@@ -4318,16 +4318,16 @@
         <v>62</v>
       </c>
       <c r="C15" s="10">
-        <v>60.1</v>
+        <v>57.35</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E15" s="10">
-        <v>54.48</v>
+        <v>47.42</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="G15" s="14" t="s">
         <v>47</v>
@@ -4342,13 +4342,13 @@
         <v>11.6</v>
       </c>
       <c r="K15" s="10">
-        <v>14.67</v>
+        <v>12.98</v>
       </c>
       <c r="L15" s="10">
-        <v>8.19</v>
+        <v>8.41</v>
       </c>
       <c r="M15" s="10">
-        <v>6.86</v>
+        <v>5.58</v>
       </c>
       <c r="N15" s="10">
         <v>4.44</v>
@@ -4368,16 +4368,16 @@
         <v>63</v>
       </c>
       <c r="C16" s="10">
-        <v>58.91</v>
+        <v>56.64</v>
       </c>
       <c r="D16" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E16" s="10">
-        <v>51.08</v>
+        <v>45.78</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="G16" s="14" t="s">
         <v>47</v>
@@ -4392,13 +4392,13 @@
         <v>11.18</v>
       </c>
       <c r="K16" s="10">
-        <v>13.35</v>
+        <v>11.95</v>
       </c>
       <c r="L16" s="10">
-        <v>8.369999999999999</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="M16" s="10">
-        <v>6.77</v>
+        <v>5.22</v>
       </c>
       <c r="N16" s="10">
         <v>6.14</v>
@@ -4418,16 +4418,16 @@
         <v>64</v>
       </c>
       <c r="C17" s="10">
-        <v>51.78</v>
+        <v>50.28</v>
       </c>
       <c r="D17" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E17" s="10">
-        <v>31.03</v>
+        <v>29.45</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G17" s="14" t="s">
         <v>10</v>
@@ -4442,13 +4442,13 @@
         <v>9.470000000000001</v>
       </c>
       <c r="K17" s="10">
-        <v>11.02</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="L17" s="10">
-        <v>8.23</v>
+        <v>8.52</v>
       </c>
       <c r="M17" s="10">
-        <v>3.36</v>
+        <v>3.06</v>
       </c>
       <c r="N17" s="10">
         <v>5.42</v>
@@ -4468,22 +4468,22 @@
         <v>65</v>
       </c>
       <c r="C18" s="10">
-        <v>50.45</v>
+        <v>47.02</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E18" s="10">
-        <v>29.31</v>
+        <v>23.54</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G18" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I18" s="10">
         <v>16.64</v>
@@ -4492,13 +4492,13 @@
         <v>4</v>
       </c>
       <c r="K18" s="10">
-        <v>11.64</v>
+        <v>10.56</v>
       </c>
       <c r="L18" s="10">
-        <v>8.06</v>
+        <v>7.28</v>
       </c>
       <c r="M18" s="10">
-        <v>6.76</v>
+        <v>5.19</v>
       </c>
       <c r="N18" s="10">
         <v>3.35</v>
@@ -4518,13 +4518,13 @@
         <v>66</v>
       </c>
       <c r="C19" s="10">
-        <v>55.45</v>
+        <v>53.7</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E19" s="10">
-        <v>44.81</v>
+        <v>42.92</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>33</v>
@@ -4542,13 +4542,13 @@
         <v>9.880000000000001</v>
       </c>
       <c r="K19" s="10">
-        <v>8.970000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="L19" s="10">
-        <v>8.210000000000001</v>
+        <v>8.09</v>
       </c>
       <c r="M19" s="10">
-        <v>6.96</v>
+        <v>5.7</v>
       </c>
       <c r="N19" s="10">
         <v>5.19</v>
@@ -4568,22 +4568,22 @@
         <v>67</v>
       </c>
       <c r="C20" s="10">
-        <v>52.65</v>
+        <v>49.74</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E20" s="10">
-        <v>37.27</v>
+        <v>33.65</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="G20" s="14" t="s">
         <v>47</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I20" s="10">
         <v>15.96</v>
@@ -4592,13 +4592,13 @@
         <v>10.15</v>
       </c>
       <c r="K20" s="10">
-        <v>7.16</v>
+        <v>7.12</v>
       </c>
       <c r="L20" s="10">
-        <v>7.91</v>
+        <v>6.38</v>
       </c>
       <c r="M20" s="10">
-        <v>7.53</v>
+        <v>6.19</v>
       </c>
       <c r="N20" s="10">
         <v>3.94</v>
@@ -4618,13 +4618,13 @@
         <v>68</v>
       </c>
       <c r="C21" s="10">
-        <v>53.91</v>
+        <v>53.13</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E21" s="10">
-        <v>41.5</v>
+        <v>42.96</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>33</v>
@@ -4642,10 +4642,10 @@
         <v>10.57</v>
       </c>
       <c r="K21" s="10">
-        <v>8.119999999999999</v>
+        <v>8.16</v>
       </c>
       <c r="L21" s="10">
-        <v>7.95</v>
+        <v>7.13</v>
       </c>
       <c r="M21" s="10">
         <v>4.73</v>
@@ -4668,16 +4668,16 @@
         <v>69</v>
       </c>
       <c r="C22" s="10">
-        <v>51.43</v>
+        <v>49.61</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E22" s="10">
-        <v>34.74</v>
+        <v>34.51</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G22" s="14" t="s">
         <v>47</v>
@@ -4692,13 +4692,13 @@
         <v>8.640000000000001</v>
       </c>
       <c r="K22" s="10">
-        <v>7.06</v>
+        <v>7.41</v>
       </c>
       <c r="L22" s="10">
-        <v>7.92</v>
+        <v>7.09</v>
       </c>
       <c r="M22" s="10">
-        <v>7.01</v>
+        <v>5.67</v>
       </c>
       <c r="N22" s="10">
         <v>4.71</v>
@@ -4718,16 +4718,16 @@
         <v>70</v>
       </c>
       <c r="C23" s="10">
-        <v>51.17</v>
+        <v>51.03</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E23" s="10">
-        <v>34.88</v>
+        <v>38.94</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="G23" s="14" t="s">
         <v>47</v>
@@ -4742,13 +4742,13 @@
         <v>10.07</v>
       </c>
       <c r="K23" s="10">
-        <v>6.66</v>
+        <v>7.1</v>
       </c>
       <c r="L23" s="10">
-        <v>7.99</v>
+        <v>7.46</v>
       </c>
       <c r="M23" s="10">
-        <v>4.67</v>
+        <v>4.62</v>
       </c>
       <c r="N23" s="10">
         <v>5.71</v>
@@ -4768,13 +4768,13 @@
         <v>71</v>
       </c>
       <c r="C24" s="10">
-        <v>55.14</v>
+        <v>55.2</v>
       </c>
       <c r="D24" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E24" s="10">
-        <v>47.09</v>
+        <v>49.86</v>
       </c>
       <c r="F24" s="14" t="s">
         <v>33</v>
@@ -4792,13 +4792,13 @@
         <v>11.07</v>
       </c>
       <c r="K24" s="10">
-        <v>6.78</v>
+        <v>7.47</v>
       </c>
       <c r="L24" s="10">
-        <v>8.699999999999999</v>
+        <v>9.34</v>
       </c>
       <c r="M24" s="10">
-        <v>6.97</v>
+        <v>5.7</v>
       </c>
       <c r="N24" s="10">
         <v>6.73</v>
@@ -4818,13 +4818,13 @@
         <v>72</v>
       </c>
       <c r="C25" s="10">
-        <v>51.72</v>
+        <v>51.98</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E25" s="10">
-        <v>37.08</v>
+        <v>41.55</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>33</v>
@@ -4833,7 +4833,7 @@
         <v>47</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I25" s="10">
         <v>14.56</v>
@@ -4842,13 +4842,13 @@
         <v>10.2</v>
       </c>
       <c r="K25" s="10">
-        <v>4.79</v>
+        <v>5.55</v>
       </c>
       <c r="L25" s="10">
-        <v>8.43</v>
+        <v>9.74</v>
       </c>
       <c r="M25" s="10">
-        <v>6.92</v>
+        <v>5.11</v>
       </c>
       <c r="N25" s="10">
         <v>6.82</v>
@@ -4868,22 +4868,22 @@
         <v>73</v>
       </c>
       <c r="C26" s="10">
-        <v>50.6</v>
+        <v>51.47</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>47</v>
       </c>
       <c r="E26" s="10">
-        <v>34.3</v>
+        <v>40.48</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="G26" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I26" s="10">
         <v>16.93</v>
@@ -4892,10 +4892,10 @@
         <v>11.43</v>
       </c>
       <c r="K26" s="10">
-        <v>4.7</v>
+        <v>5.79</v>
       </c>
       <c r="L26" s="10">
-        <v>8.609999999999999</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="M26" s="10">
         <v>4.89</v>
@@ -4918,22 +4918,22 @@
         <v>74</v>
       </c>
       <c r="C27" s="10">
-        <v>44.66</v>
+        <v>44.38</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E27" s="10">
-        <v>17.43</v>
+        <v>21.85</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G27" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I27" s="10">
         <v>12.61</v>
@@ -4942,13 +4942,13 @@
         <v>8.08</v>
       </c>
       <c r="K27" s="10">
-        <v>2.48</v>
+        <v>2.55</v>
       </c>
       <c r="L27" s="10">
-        <v>8.82</v>
+        <v>9.77</v>
       </c>
       <c r="M27" s="10">
-        <v>7</v>
+        <v>5.7</v>
       </c>
       <c r="N27" s="10">
         <v>5.67</v>
@@ -4968,22 +4968,22 @@
         <v>75</v>
       </c>
       <c r="C28" s="10">
-        <v>47.92</v>
+        <v>46.59</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E28" s="10">
-        <v>30.18</v>
+        <v>30.12</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I28" s="10">
         <v>15.32</v>
@@ -4992,13 +4992,13 @@
         <v>8.35</v>
       </c>
       <c r="K28" s="10">
-        <v>4.36</v>
+        <v>4.92</v>
       </c>
       <c r="L28" s="10">
-        <v>8.609999999999999</v>
+        <v>8.19</v>
       </c>
       <c r="M28" s="10">
-        <v>6.86</v>
+        <v>5.39</v>
       </c>
       <c r="N28" s="10">
         <v>4.42</v>
@@ -5018,16 +5018,16 @@
         <v>76</v>
       </c>
       <c r="C29" s="10">
-        <v>47.2</v>
+        <v>47.67</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>33</v>
       </c>
       <c r="E29" s="10">
-        <v>29.37</v>
+        <v>33.97</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>10</v>
@@ -5042,13 +5042,13 @@
         <v>7.28</v>
       </c>
       <c r="K29" s="10">
-        <v>8.57</v>
+        <v>8.08</v>
       </c>
       <c r="L29" s="10">
-        <v>8.24</v>
+        <v>7.63</v>
       </c>
       <c r="M29" s="10">
-        <v>2.59</v>
+        <v>4.16</v>
       </c>
       <c r="N29" s="10">
         <v>6.04</v>
@@ -5539,7 +5539,7 @@
         <v>53</v>
       </c>
       <c r="H40" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I40" s="7" t="s">
         <v>57</v>
@@ -7667,8 +7667,8 @@
       <c r="E25" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="F25" s="14" t="s">
-        <v>94</v>
+      <c r="F25" s="10">
+        <v>39.7</v>
       </c>
       <c r="G25" s="17" t="s">
         <v>187</v>
@@ -7687,8 +7687,8 @@
       <c r="E26" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="F26" s="14" t="s">
-        <v>94</v>
+      <c r="F26" s="10">
+        <v>42.5</v>
       </c>
       <c r="G26" s="17" t="s">
         <v>187</v>
@@ -7874,7 +7874,7 @@
         <v>241</v>
       </c>
       <c r="C6" s="16">
-        <v>0.1483538183721982</v>
+        <v>0.2837804645096819</v>
       </c>
     </row>
     <row r="7" spans="2:3">
@@ -7882,7 +7882,7 @@
         <v>242</v>
       </c>
       <c r="C7" s="16">
-        <v>0.1067193675889328</v>
+        <v>0.251270468661773</v>
       </c>
     </row>
     <row r="8" spans="2:3">
@@ -7890,7 +7890,7 @@
         <v>243</v>
       </c>
       <c r="C8" s="16">
-        <v>0.05631062061483348</v>
+        <v>0.03964834070416489</v>
       </c>
     </row>
     <row r="9" spans="2:3">
@@ -7898,7 +7898,7 @@
         <v>244</v>
       </c>
       <c r="C9" s="16">
-        <v>0.0378424189052429</v>
+        <v>-0.0254093732354602</v>
       </c>
     </row>
     <row r="10" spans="2:3">
@@ -7914,7 +7914,7 @@
         <v>246</v>
       </c>
       <c r="C11" s="11">
-        <v>0.5454545454545454</v>
+        <v>0.5909090909090909</v>
       </c>
     </row>
     <row r="12" spans="2:3">
@@ -7922,7 +7922,7 @@
         <v>247</v>
       </c>
       <c r="C12" s="11">
-        <v>0.1729797086322691</v>
+        <v>0.3017843613374662</v>
       </c>
     </row>
     <row r="13" spans="2:3">
@@ -7930,7 +7930,7 @@
         <v>248</v>
       </c>
       <c r="C13" s="11">
-        <v>0.306871980645762</v>
+        <v>0.3056281529812772</v>
       </c>
     </row>
     <row r="14" spans="2:3">
@@ -7946,7 +7946,7 @@
         <v>250</v>
       </c>
       <c r="C15" s="10">
-        <v>0.4192135232141344</v>
+        <v>0.6829570846962959</v>
       </c>
     </row>
     <row r="16" spans="2:3">
@@ -8001,13 +8001,13 @@
         <v>47</v>
       </c>
       <c r="C21" s="14">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D21" s="11">
-        <v>0.02110257050780219</v>
+        <v>0.02931877005550193</v>
       </c>
       <c r="E21" s="11">
-        <v>0.0131170626569212</v>
+        <v>0.02403825543019816</v>
       </c>
       <c r="F21" s="11">
         <v>0.5</v>
@@ -8018,33 +8018,33 @@
         <v>33</v>
       </c>
       <c r="C22" s="14">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D22" s="11">
-        <v>-0.03516352497855219</v>
+        <v>0.03282067277409505</v>
       </c>
       <c r="E22" s="11">
-        <v>-0.01642933677034653</v>
+        <v>0.03163927438071323</v>
       </c>
       <c r="F22" s="11">
-        <v>0.4285714285714285</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="23" spans="2:12">
       <c r="B23" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C23" s="14">
         <v>8</v>
       </c>
       <c r="D23" s="11">
-        <v>0.05467139182258603</v>
+        <v>-0.01185240655140339</v>
       </c>
       <c r="E23" s="11">
-        <v>0.05505192201341436</v>
+        <v>-0.02331096225865564</v>
       </c>
       <c r="F23" s="11">
-        <v>0.625</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="25" spans="2:12">
@@ -8092,7 +8092,7 @@
         <v>45</v>
       </c>
       <c r="C27" s="10">
-        <v>68.64</v>
+        <v>66.86</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>46</v>
@@ -8101,7 +8101,7 @@
         <v>0.775</v>
       </c>
       <c r="F27" s="10">
-        <v>68.64</v>
+        <v>66.86</v>
       </c>
       <c r="G27" s="14" t="s">
         <v>46</v>
@@ -8127,7 +8127,7 @@
         <v>50</v>
       </c>
       <c r="C28" s="10">
-        <v>60.11</v>
+        <v>62.75</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>47</v>
@@ -8136,7 +8136,7 @@
         <v>0.5</v>
       </c>
       <c r="F28" s="10">
-        <v>60.11</v>
+        <v>62.75</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>47</v>
@@ -8162,7 +8162,7 @@
         <v>51</v>
       </c>
       <c r="C29" s="10">
-        <v>60.26</v>
+        <v>63.44</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>47</v>
@@ -8171,7 +8171,7 @@
         <v>0.5</v>
       </c>
       <c r="F29" s="10">
-        <v>60.26</v>
+        <v>63.44</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>47</v>
@@ -8197,7 +8197,7 @@
         <v>52</v>
       </c>
       <c r="C30" s="10">
-        <v>57.42</v>
+        <v>60.22</v>
       </c>
       <c r="D30" s="14" t="s">
         <v>47</v>
@@ -8206,7 +8206,7 @@
         <v>0.5</v>
       </c>
       <c r="F30" s="10">
-        <v>57.42</v>
+        <v>60.22</v>
       </c>
       <c r="G30" s="14" t="s">
         <v>47</v>
@@ -8232,16 +8232,16 @@
         <v>53</v>
       </c>
       <c r="C31" s="10">
-        <v>45.35</v>
+        <v>30.12</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="E31" s="9">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="F31" s="10">
-        <v>60.1</v>
+        <v>59.69</v>
       </c>
       <c r="G31" s="14" t="s">
         <v>47</v>
@@ -8250,13 +8250,13 @@
         <v>-0.197399725228697</v>
       </c>
       <c r="I31" s="11">
-        <v>-0.05921991756860909</v>
+        <v>-0.0197399725228697</v>
       </c>
       <c r="J31" s="17" t="s">
         <v>267</v>
       </c>
       <c r="K31" s="10">
-        <v>110.7044130913189</v>
+        <v>115.3501365996978</v>
       </c>
       <c r="L31" s="10">
         <v>100.5170214194588</v>
@@ -8264,19 +8264,19 @@
     </row>
     <row r="32" spans="2:12">
       <c r="B32" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C32" s="10">
-        <v>11.29</v>
+        <v>0</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E32" s="9">
         <v>0.1</v>
       </c>
       <c r="F32" s="10">
-        <v>50.29</v>
+        <v>51.25</v>
       </c>
       <c r="G32" s="14" t="s">
         <v>47</v>
@@ -8291,7 +8291,7 @@
         <v>267</v>
       </c>
       <c r="K32" s="10">
-        <v>110.0990329966838</v>
+        <v>114.7193516593242</v>
       </c>
       <c r="L32" s="10">
         <v>95.02031155576445</v>
@@ -8302,7 +8302,7 @@
         <v>57</v>
       </c>
       <c r="C33" s="10">
-        <v>46.77</v>
+        <v>40.99</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>33</v>
@@ -8311,7 +8311,7 @@
         <v>0.3</v>
       </c>
       <c r="F33" s="10">
-        <v>58.2</v>
+        <v>57.52</v>
       </c>
       <c r="G33" s="14" t="s">
         <v>47</v>
@@ -8326,7 +8326,7 @@
         <v>267</v>
       </c>
       <c r="K33" s="10">
-        <v>106.4515302526274</v>
+        <v>110.9187810404491</v>
       </c>
       <c r="L33" s="10">
         <v>84.52712683811188</v>
@@ -8337,16 +8337,16 @@
         <v>59</v>
       </c>
       <c r="C34" s="10">
-        <v>20.65</v>
+        <v>6.74</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E34" s="9">
         <v>0.1</v>
       </c>
       <c r="F34" s="10">
-        <v>48.71</v>
+        <v>45.88</v>
       </c>
       <c r="G34" s="14" t="s">
         <v>33</v>
@@ -8361,7 +8361,7 @@
         <v>268</v>
       </c>
       <c r="K34" s="10">
-        <v>107.0598458516343</v>
+        <v>111.5526246739752</v>
       </c>
       <c r="L34" s="10">
         <v>89.35741623581549</v>
@@ -8372,7 +8372,7 @@
         <v>60</v>
       </c>
       <c r="C35" s="10">
-        <v>57.76</v>
+        <v>50.08</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>47</v>
@@ -8381,7 +8381,7 @@
         <v>0.5</v>
       </c>
       <c r="F35" s="10">
-        <v>61.2</v>
+        <v>58.49</v>
       </c>
       <c r="G35" s="14" t="s">
         <v>47</v>
@@ -8396,7 +8396,7 @@
         <v>267</v>
       </c>
       <c r="K35" s="10">
-        <v>109.8523878557859</v>
+        <v>114.4623560265416</v>
       </c>
       <c r="L35" s="10">
         <v>94.01900221580608</v>
@@ -8407,16 +8407,16 @@
         <v>62</v>
       </c>
       <c r="C36" s="10">
-        <v>54.48</v>
+        <v>47.42</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E36" s="9">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="F36" s="10">
-        <v>60.1</v>
+        <v>57.35</v>
       </c>
       <c r="G36" s="14" t="s">
         <v>47</v>
@@ -8425,13 +8425,13 @@
         <v>0.03032548340445285</v>
       </c>
       <c r="I36" s="11">
-        <v>0.01516274170222642</v>
-      </c>
-      <c r="J36" s="17" t="s">
-        <v>267</v>
+        <v>0.009097645021335853</v>
+      </c>
+      <c r="J36" s="13" t="s">
+        <v>268</v>
       </c>
       <c r="K36" s="10">
-        <v>111.518051238216</v>
+        <v>115.5036939099769</v>
       </c>
       <c r="L36" s="10">
         <v>96.87017390720473</v>
@@ -8442,16 +8442,16 @@
         <v>63</v>
       </c>
       <c r="C37" s="10">
-        <v>51.08</v>
+        <v>45.78</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="E37" s="9">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="F37" s="10">
-        <v>58.91</v>
+        <v>56.64</v>
       </c>
       <c r="G37" s="14" t="s">
         <v>47</v>
@@ -8460,13 +8460,13 @@
         <v>-0.0209851405796474</v>
       </c>
       <c r="I37" s="11">
-        <v>-0.0104925702898237</v>
-      </c>
-      <c r="J37" s="13" t="s">
-        <v>268</v>
+        <v>-0.00629554217389422</v>
+      </c>
+      <c r="J37" s="17" t="s">
+        <v>267</v>
       </c>
       <c r="K37" s="10">
-        <v>110.3479402470148</v>
+        <v>114.7765355337261</v>
       </c>
       <c r="L37" s="10">
         <v>94.83733968978714</v>
@@ -8477,16 +8477,16 @@
         <v>64</v>
       </c>
       <c r="C38" s="10">
-        <v>31.03</v>
+        <v>29.45</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E38" s="9">
         <v>0.1</v>
       </c>
       <c r="F38" s="10">
-        <v>51.78</v>
+        <v>50.28</v>
       </c>
       <c r="G38" s="14" t="s">
         <v>47</v>
@@ -8501,7 +8501,7 @@
         <v>268</v>
       </c>
       <c r="K38" s="10">
-        <v>111.8534528423508</v>
+        <v>116.3424688851619</v>
       </c>
       <c r="L38" s="10">
         <v>107.7763043040354</v>
@@ -8512,19 +8512,19 @@
         <v>65</v>
       </c>
       <c r="C39" s="10">
-        <v>29.31</v>
+        <v>23.54</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E39" s="9">
         <v>0.1</v>
       </c>
       <c r="F39" s="10">
-        <v>50.45</v>
+        <v>47.02</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="H39" s="11">
         <v>-0.03019258774696476</v>
@@ -8536,7 +8536,7 @@
         <v>267</v>
       </c>
       <c r="K39" s="10">
-        <v>111.5157383233764</v>
+        <v>115.9912008651105</v>
       </c>
       <c r="L39" s="10">
         <v>104.5222587792923</v>
@@ -8547,7 +8547,7 @@
         <v>66</v>
       </c>
       <c r="C40" s="10">
-        <v>44.81</v>
+        <v>42.92</v>
       </c>
       <c r="D40" s="14" t="s">
         <v>33</v>
@@ -8556,7 +8556,7 @@
         <v>0.3</v>
       </c>
       <c r="F40" s="10">
-        <v>55.45</v>
+        <v>53.7</v>
       </c>
       <c r="G40" s="14" t="s">
         <v>47</v>
@@ -8571,7 +8571,7 @@
         <v>268</v>
       </c>
       <c r="K40" s="10">
-        <v>112.6606972336988</v>
+        <v>117.1821104259152</v>
       </c>
       <c r="L40" s="10">
         <v>108.0994426911972</v>
@@ -8582,31 +8582,31 @@
         <v>67</v>
       </c>
       <c r="C41" s="10">
-        <v>37.27</v>
+        <v>33.65</v>
       </c>
       <c r="D41" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E41" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="F41" s="10">
+        <v>49.74</v>
+      </c>
+      <c r="G41" s="14" t="s">
         <v>33</v>
-      </c>
-      <c r="E41" s="9">
-        <v>0.3</v>
-      </c>
-      <c r="F41" s="10">
-        <v>52.65</v>
-      </c>
-      <c r="G41" s="14" t="s">
-        <v>47</v>
       </c>
       <c r="H41" s="11">
         <v>-0.01642933677034653</v>
       </c>
       <c r="I41" s="11">
-        <v>-0.004928801031103957</v>
+        <v>-0.001642933677034653</v>
       </c>
       <c r="J41" s="17" t="s">
         <v>267</v>
       </c>
       <c r="K41" s="10">
-        <v>112.1054150730085</v>
+        <v>116.9895879903505</v>
       </c>
       <c r="L41" s="10">
         <v>106.3234405425367</v>
@@ -8617,7 +8617,7 @@
         <v>68</v>
       </c>
       <c r="C42" s="10">
-        <v>41.5</v>
+        <v>42.96</v>
       </c>
       <c r="D42" s="14" t="s">
         <v>33</v>
@@ -8626,7 +8626,7 @@
         <v>0.3</v>
       </c>
       <c r="F42" s="10">
-        <v>53.91</v>
+        <v>53.13</v>
       </c>
       <c r="G42" s="14" t="s">
         <v>47</v>
@@ -8641,7 +8641,7 @@
         <v>268</v>
       </c>
       <c r="K42" s="10">
-        <v>113.1694952691261</v>
+        <v>118.1000276925845</v>
       </c>
       <c r="L42" s="10">
         <v>109.6874370509635</v>
@@ -8652,19 +8652,19 @@
         <v>69</v>
       </c>
       <c r="C43" s="10">
-        <v>34.74</v>
+        <v>34.51</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E43" s="9">
         <v>0.1</v>
       </c>
       <c r="F43" s="10">
-        <v>51.43</v>
+        <v>49.61</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="H43" s="11">
         <v>0.05295900096414319</v>
@@ -8676,7 +8676,7 @@
         <v>268</v>
       </c>
       <c r="K43" s="10">
-        <v>113.768829610033</v>
+        <v>118.7254736406282</v>
       </c>
       <c r="L43" s="10">
         <v>115.4963741354999</v>
@@ -8687,16 +8687,16 @@
         <v>70</v>
       </c>
       <c r="C44" s="10">
-        <v>34.88</v>
+        <v>38.94</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E44" s="9">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="F44" s="10">
-        <v>51.17</v>
+        <v>51.03</v>
       </c>
       <c r="G44" s="14" t="s">
         <v>47</v>
@@ -8705,13 +8705,13 @@
         <v>0.2075693823715363</v>
       </c>
       <c r="I44" s="11">
-        <v>0.02075693823715363</v>
+        <v>0.0622708147114609</v>
       </c>
       <c r="J44" s="13" t="s">
         <v>268</v>
       </c>
       <c r="K44" s="10">
-        <v>116.1303221795618</v>
+        <v>126.1186056112342</v>
       </c>
       <c r="L44" s="10">
         <v>139.4698851809575</v>
@@ -8722,7 +8722,7 @@
         <v>71</v>
       </c>
       <c r="C45" s="10">
-        <v>47.09</v>
+        <v>49.86</v>
       </c>
       <c r="D45" s="14" t="s">
         <v>33</v>
@@ -8731,7 +8731,7 @@
         <v>0.3</v>
       </c>
       <c r="F45" s="10">
-        <v>55.14</v>
+        <v>55.2</v>
       </c>
       <c r="G45" s="14" t="s">
         <v>47</v>
@@ -8746,7 +8746,7 @@
         <v>268</v>
       </c>
       <c r="K45" s="10">
-        <v>118.7047295203143</v>
+        <v>128.9144358302274</v>
       </c>
       <c r="L45" s="10">
         <v>149.7759014302021</v>
@@ -8757,7 +8757,7 @@
         <v>72</v>
       </c>
       <c r="C46" s="10">
-        <v>37.08</v>
+        <v>41.55</v>
       </c>
       <c r="D46" s="14" t="s">
         <v>33</v>
@@ -8766,7 +8766,7 @@
         <v>0.3</v>
       </c>
       <c r="F46" s="10">
-        <v>51.72</v>
+        <v>51.98</v>
       </c>
       <c r="G46" s="14" t="s">
         <v>47</v>
@@ -8781,7 +8781,7 @@
         <v>267</v>
       </c>
       <c r="K46" s="10">
-        <v>116.5095611113177</v>
+        <v>126.5304626040409</v>
       </c>
       <c r="L46" s="10">
         <v>140.5433760827234</v>
@@ -8792,16 +8792,16 @@
         <v>73</v>
       </c>
       <c r="C47" s="10">
-        <v>34.3</v>
+        <v>40.48</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E47" s="9">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="F47" s="10">
-        <v>50.6</v>
+        <v>51.47</v>
       </c>
       <c r="G47" s="14" t="s">
         <v>47</v>
@@ -8810,13 +8810,13 @@
         <v>0.1107919426213355</v>
       </c>
       <c r="I47" s="11">
-        <v>0.01107919426213355</v>
+        <v>0.03323758278640065</v>
       </c>
       <c r="J47" s="13" t="s">
         <v>268</v>
       </c>
       <c r="K47" s="10">
-        <v>117.8003931722659</v>
+        <v>130.7360293298443</v>
       </c>
       <c r="L47" s="10">
         <v>156.1144497414892</v>
@@ -8827,16 +8827,16 @@
         <v>74</v>
       </c>
       <c r="C48" s="10">
-        <v>17.43</v>
+        <v>21.85</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E48" s="9">
         <v>0.1</v>
       </c>
       <c r="F48" s="10">
-        <v>44.66</v>
+        <v>44.38</v>
       </c>
       <c r="G48" s="14" t="s">
         <v>33</v>
@@ -8851,7 +8851,7 @@
         <v>267</v>
       </c>
       <c r="K48" s="10">
-        <v>117.2979708632269</v>
+        <v>130.1784361337466</v>
       </c>
       <c r="L48" s="10">
         <v>149.4561203249849</v>

</xml_diff>